<commit_message>
feat(ui): consolidate site tab entry and implement smart inventory import
</commit_message>
<xml_diff>
--- a/data/Material_Inventory.xlsx
+++ b/data/Material_Inventory.xlsx
@@ -20872,7 +20872,7 @@
         <v>0</v>
       </c>
       <c r="S405" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="406">
@@ -20925,7 +20925,7 @@
         <v>1000</v>
       </c>
       <c r="S406" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="407">
@@ -20976,7 +20976,7 @@
         <v>0</v>
       </c>
       <c r="S407" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="408">
@@ -21019,7 +21019,7 @@
         <v>0</v>
       </c>
       <c r="S408" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="409">
@@ -21062,7 +21062,7 @@
         <v>0</v>
       </c>
       <c r="S409" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="410">
@@ -21105,7 +21105,7 @@
         <v>0</v>
       </c>
       <c r="S410" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="411">
@@ -21148,7 +21148,7 @@
         <v>0</v>
       </c>
       <c r="S411" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="412">
@@ -21188,7 +21188,9 @@
         <v>5</v>
       </c>
       <c r="R412" t="inlineStr"/>
-      <c r="S412" t="inlineStr"/>
+      <c r="S412" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="413">
       <c r="A413" t="n">
@@ -21227,7 +21229,9 @@
         <v>10</v>
       </c>
       <c r="R413" t="inlineStr"/>
-      <c r="S413" t="inlineStr"/>
+      <c r="S413" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="414">
       <c r="A414" t="n">
@@ -21266,7 +21270,9 @@
         <v>5</v>
       </c>
       <c r="R414" t="inlineStr"/>
-      <c r="S414" t="inlineStr"/>
+      <c r="S414" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="415">
       <c r="A415" t="n">
@@ -21305,7 +21311,9 @@
         <v>10</v>
       </c>
       <c r="R415" t="inlineStr"/>
-      <c r="S415" t="inlineStr"/>
+      <c r="S415" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="416">
       <c r="A416" t="n">
@@ -21344,7 +21352,9 @@
         <v>10</v>
       </c>
       <c r="R416" t="inlineStr"/>
-      <c r="S416" t="inlineStr"/>
+      <c r="S416" t="n">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -21357,7 +21367,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21416,6 +21426,37 @@
           <t>차량비고</t>
         </is>
       </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="n">
+        <v>46127.83419630787</v>
+      </c>
+      <c r="B2" t="n">
+        <v>410</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>-200</v>
+      </c>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>부장 주진철</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>K1-PJT</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat: enhance daily usage save logic for multiple companies and UI stability fixes
</commit_message>
<xml_diff>
--- a/data/Material_Inventory.xlsx
+++ b/data/Material_Inventory.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Materials" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Transactions" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="MonthlyUsage" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="DailyUsage" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Budget" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Materials" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Transactions" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MonthlyUsage" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DailyUsage" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S416"/>
+  <dimension ref="A1:S419"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21354,6 +21354,153 @@
       <c r="R416" t="inlineStr"/>
       <c r="S416" t="n">
         <v>0</v>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="n">
+        <v>418</v>
+      </c>
+      <c r="B417" t="inlineStr"/>
+      <c r="C417" t="inlineStr"/>
+      <c r="D417" t="inlineStr">
+        <is>
+          <t>PT약품</t>
+        </is>
+      </c>
+      <c r="E417" t="inlineStr"/>
+      <c r="F417" t="inlineStr">
+        <is>
+          <t>세척제</t>
+        </is>
+      </c>
+      <c r="G417" t="inlineStr"/>
+      <c r="H417" t="inlineStr"/>
+      <c r="I417" t="inlineStr">
+        <is>
+          <t>NAWOO</t>
+        </is>
+      </c>
+      <c r="J417" t="inlineStr"/>
+      <c r="K417" t="n">
+        <v>0</v>
+      </c>
+      <c r="L417" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="M417" t="n">
+        <v>0</v>
+      </c>
+      <c r="N417" t="inlineStr"/>
+      <c r="O417" t="inlineStr"/>
+      <c r="P417" t="inlineStr"/>
+      <c r="Q417" t="n">
+        <v>0</v>
+      </c>
+      <c r="R417" t="n">
+        <v>0</v>
+      </c>
+      <c r="S417" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="n">
+        <v>419</v>
+      </c>
+      <c r="B418" t="inlineStr"/>
+      <c r="C418" t="inlineStr"/>
+      <c r="D418" t="inlineStr">
+        <is>
+          <t>PT약품</t>
+        </is>
+      </c>
+      <c r="E418" t="inlineStr"/>
+      <c r="F418" t="inlineStr">
+        <is>
+          <t>침투제</t>
+        </is>
+      </c>
+      <c r="G418" t="inlineStr"/>
+      <c r="H418" t="inlineStr"/>
+      <c r="I418" t="inlineStr">
+        <is>
+          <t>NAWOO</t>
+        </is>
+      </c>
+      <c r="J418" t="inlineStr"/>
+      <c r="K418" t="n">
+        <v>0</v>
+      </c>
+      <c r="L418" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="M418" t="n">
+        <v>0</v>
+      </c>
+      <c r="N418" t="inlineStr"/>
+      <c r="O418" t="inlineStr"/>
+      <c r="P418" t="inlineStr"/>
+      <c r="Q418" t="n">
+        <v>0</v>
+      </c>
+      <c r="R418" t="n">
+        <v>0</v>
+      </c>
+      <c r="S418" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="n">
+        <v>420</v>
+      </c>
+      <c r="B419" t="inlineStr"/>
+      <c r="C419" t="inlineStr"/>
+      <c r="D419" t="inlineStr">
+        <is>
+          <t>PT약품</t>
+        </is>
+      </c>
+      <c r="E419" t="inlineStr"/>
+      <c r="F419" t="inlineStr">
+        <is>
+          <t>현상제</t>
+        </is>
+      </c>
+      <c r="G419" t="inlineStr"/>
+      <c r="H419" t="inlineStr"/>
+      <c r="I419" t="inlineStr">
+        <is>
+          <t>NAWOO</t>
+        </is>
+      </c>
+      <c r="J419" t="inlineStr"/>
+      <c r="K419" t="n">
+        <v>0</v>
+      </c>
+      <c r="L419" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="M419" t="n">
+        <v>0</v>
+      </c>
+      <c r="N419" t="inlineStr"/>
+      <c r="O419" t="inlineStr"/>
+      <c r="P419" t="inlineStr"/>
+      <c r="Q419" t="n">
+        <v>0</v>
+      </c>
+      <c r="R419" t="n">
+        <v>0</v>
+      </c>
+      <c r="S419" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refine Site and Monthly tabs: restricted items to history, defaulted filters to 'All', added worker summary auto-hiding, and unified hyphenated site names
</commit_message>
<xml_diff>
--- a/data/Material_Inventory.xlsx
+++ b/data/Material_Inventory.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Materials" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Transactions" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MonthlyUsage" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DailyUsage" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Materials" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Transactions" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="MonthlyUsage" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="DailyUsage" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Budget" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S419"/>
+  <dimension ref="A1:S422"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21105,7 +21105,7 @@
         <v>0</v>
       </c>
       <c r="S410" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="411">
@@ -21402,7 +21402,7 @@
         <v>0</v>
       </c>
       <c r="S417" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="418">
@@ -21451,7 +21451,7 @@
         <v>0</v>
       </c>
       <c r="S418" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="419">
@@ -21500,6 +21500,165 @@
         <v>0</v>
       </c>
       <c r="S419" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" t="n">
+        <v>421</v>
+      </c>
+      <c r="B420" t="inlineStr"/>
+      <c r="C420" t="inlineStr"/>
+      <c r="D420" t="inlineStr">
+        <is>
+          <t>MT약품</t>
+        </is>
+      </c>
+      <c r="E420" t="inlineStr">
+        <is>
+          <t>현장</t>
+        </is>
+      </c>
+      <c r="F420" t="inlineStr">
+        <is>
+          <t>MT약품</t>
+        </is>
+      </c>
+      <c r="G420" t="inlineStr">
+        <is>
+          <t>자동등록</t>
+        </is>
+      </c>
+      <c r="H420" t="inlineStr"/>
+      <c r="I420" t="inlineStr"/>
+      <c r="J420" t="inlineStr"/>
+      <c r="K420" t="n">
+        <v>0</v>
+      </c>
+      <c r="L420" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="M420" t="n">
+        <v>0</v>
+      </c>
+      <c r="N420" t="inlineStr"/>
+      <c r="O420" t="inlineStr"/>
+      <c r="P420" t="inlineStr"/>
+      <c r="Q420" t="n">
+        <v>10</v>
+      </c>
+      <c r="R420" t="n">
+        <v>0</v>
+      </c>
+      <c r="S420" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" t="n">
+        <v>422</v>
+      </c>
+      <c r="B421" t="inlineStr"/>
+      <c r="C421" t="inlineStr"/>
+      <c r="D421" t="inlineStr">
+        <is>
+          <t>MT약품</t>
+        </is>
+      </c>
+      <c r="E421" t="inlineStr">
+        <is>
+          <t>현장</t>
+        </is>
+      </c>
+      <c r="F421" t="inlineStr">
+        <is>
+          <t>흑색자분</t>
+        </is>
+      </c>
+      <c r="G421" t="inlineStr">
+        <is>
+          <t>자동등록</t>
+        </is>
+      </c>
+      <c r="H421" t="inlineStr"/>
+      <c r="I421" t="inlineStr"/>
+      <c r="J421" t="inlineStr"/>
+      <c r="K421" t="n">
+        <v>0</v>
+      </c>
+      <c r="L421" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="M421" t="n">
+        <v>0</v>
+      </c>
+      <c r="N421" t="inlineStr"/>
+      <c r="O421" t="inlineStr"/>
+      <c r="P421" t="inlineStr"/>
+      <c r="Q421" t="n">
+        <v>10</v>
+      </c>
+      <c r="R421" t="n">
+        <v>0</v>
+      </c>
+      <c r="S421" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" t="n">
+        <v>423</v>
+      </c>
+      <c r="B422" t="inlineStr"/>
+      <c r="C422" t="inlineStr"/>
+      <c r="D422" t="inlineStr">
+        <is>
+          <t>MT약품</t>
+        </is>
+      </c>
+      <c r="E422" t="inlineStr">
+        <is>
+          <t>현장</t>
+        </is>
+      </c>
+      <c r="F422" t="inlineStr">
+        <is>
+          <t>백색페인트</t>
+        </is>
+      </c>
+      <c r="G422" t="inlineStr">
+        <is>
+          <t>자동등록</t>
+        </is>
+      </c>
+      <c r="H422" t="inlineStr"/>
+      <c r="I422" t="inlineStr"/>
+      <c r="J422" t="inlineStr"/>
+      <c r="K422" t="n">
+        <v>0</v>
+      </c>
+      <c r="L422" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="M422" t="n">
+        <v>0</v>
+      </c>
+      <c r="N422" t="inlineStr"/>
+      <c r="O422" t="inlineStr"/>
+      <c r="P422" t="inlineStr"/>
+      <c r="Q422" t="n">
+        <v>10</v>
+      </c>
+      <c r="R422" t="n">
+        <v>0</v>
+      </c>
+      <c r="S422" t="n">
         <v>1</v>
       </c>
     </row>
@@ -21514,7 +21673,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21573,37 +21732,6 @@
           <t>차량비고</t>
         </is>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="1" t="n">
-        <v>46127.83419630787</v>
-      </c>
-      <c r="B2" t="n">
-        <v>410</v>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>OUT</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>-200</v>
-      </c>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>부장 주진철</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>K1-PJT</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -21667,7 +21795,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BK4"/>
+  <dimension ref="A1:BM4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21984,6 +22112,16 @@
       <c r="BK1" t="inlineStr">
         <is>
           <t>차량비고</t>
+        </is>
+      </c>
+      <c r="BL1" t="inlineStr">
+        <is>
+          <t>RTK_총계</t>
+        </is>
+      </c>
+      <c r="BM1" t="inlineStr">
+        <is>
+          <t>회사코드</t>
         </is>
       </c>
     </row>
@@ -22135,6 +22273,8 @@
       <c r="BI2" t="inlineStr"/>
       <c r="BJ2" t="inlineStr"/>
       <c r="BK2" t="inlineStr"/>
+      <c r="BL2" t="inlineStr"/>
+      <c r="BM2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr"/>
@@ -22308,6 +22448,8 @@
         </is>
       </c>
       <c r="BK3" t="inlineStr"/>
+      <c r="BL3" t="inlineStr"/>
+      <c r="BM3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr"/>
@@ -22481,6 +22623,8 @@
         </is>
       </c>
       <c r="BK4" t="inlineStr"/>
+      <c r="BL4" t="inlineStr"/>
+      <c r="BM4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat: Implement Unified Global Session Save/Load and enhance Site tab UI
</commit_message>
<xml_diff>
--- a/data/Material_Inventory.xlsx
+++ b/data/Material_Inventory.xlsx
@@ -21673,7 +21673,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21730,6 +21730,57 @@
       <c r="K1" t="inlineStr">
         <is>
           <t>차량비고</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="n">
+        <v>46131</v>
+      </c>
+      <c r="B2" t="n">
+        <v>410</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>-25</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>K1-PJT 현장 사용 (자동 차감)</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>부장 주진철, 주임 김진환</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>K1-PJT</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>nan</t>
         </is>
       </c>
     </row>
@@ -21795,7 +21846,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BM4"/>
+  <dimension ref="A1:BN5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22122,6 +22173,11 @@
       <c r="BM1" t="inlineStr">
         <is>
           <t>회사코드</t>
+        </is>
+      </c>
+      <c r="BN1" t="inlineStr">
+        <is>
+          <t>업체명</t>
         </is>
       </c>
     </row>
@@ -22275,6 +22331,7 @@
       <c r="BK2" t="inlineStr"/>
       <c r="BL2" t="inlineStr"/>
       <c r="BM2" t="inlineStr"/>
+      <c r="BN2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr"/>
@@ -22450,6 +22507,7 @@
       <c r="BK3" t="inlineStr"/>
       <c r="BL3" t="inlineStr"/>
       <c r="BM3" t="inlineStr"/>
+      <c r="BN3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr"/>
@@ -22625,6 +22683,165 @@
       <c r="BK4" t="inlineStr"/>
       <c r="BL4" t="inlineStr"/>
       <c r="BM4" t="inlineStr"/>
+      <c r="BN4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="n">
+        <v>46131</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>K1-PJT</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>410</v>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" s="1" t="n">
+        <v>46131.88805793982</v>
+      </c>
+      <c r="G5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="n">
+        <v>1</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>부장 주진철</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>R-RAY</t>
+        </is>
+      </c>
+      <c r="P5" t="n">
+        <v>25</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>25500</v>
+      </c>
+      <c r="R5" t="n">
+        <v>0</v>
+      </c>
+      <c r="S5" t="n">
+        <v>0</v>
+      </c>
+      <c r="T5" t="n">
+        <v>0</v>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>RT</t>
+        </is>
+      </c>
+      <c r="V5" t="n">
+        <v>0</v>
+      </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>09:00~20:00</t>
+        </is>
+      </c>
+      <c r="X5" t="inlineStr">
+        <is>
+          <t>82,500</t>
+        </is>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>주임 김진환</t>
+        </is>
+      </c>
+      <c r="Z5" t="inlineStr">
+        <is>
+          <t>09:00~20:00</t>
+        </is>
+      </c>
+      <c r="AA5" t="inlineStr">
+        <is>
+          <t>82,500</t>
+        </is>
+      </c>
+      <c r="AB5" t="inlineStr"/>
+      <c r="AC5" t="inlineStr"/>
+      <c r="AD5" t="inlineStr"/>
+      <c r="AE5" t="inlineStr"/>
+      <c r="AF5" t="inlineStr"/>
+      <c r="AG5" t="inlineStr"/>
+      <c r="AH5" t="inlineStr"/>
+      <c r="AI5" t="inlineStr"/>
+      <c r="AJ5" t="inlineStr"/>
+      <c r="AK5" t="inlineStr"/>
+      <c r="AL5" t="inlineStr"/>
+      <c r="AM5" t="inlineStr"/>
+      <c r="AN5" t="inlineStr"/>
+      <c r="AO5" t="inlineStr"/>
+      <c r="AP5" t="inlineStr"/>
+      <c r="AQ5" t="inlineStr"/>
+      <c r="AR5" t="inlineStr"/>
+      <c r="AS5" t="inlineStr"/>
+      <c r="AT5" t="inlineStr"/>
+      <c r="AU5" t="inlineStr"/>
+      <c r="AV5" t="inlineStr"/>
+      <c r="AW5" t="inlineStr"/>
+      <c r="AX5" t="inlineStr"/>
+      <c r="AY5" t="inlineStr"/>
+      <c r="AZ5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH5" t="inlineStr"/>
+      <c r="BI5" t="inlineStr"/>
+      <c r="BJ5" t="inlineStr"/>
+      <c r="BK5" t="inlineStr"/>
+      <c r="BL5" t="n">
+        <v>2</v>
+      </c>
+      <c r="BM5" t="inlineStr"/>
+      <c r="BN5" t="inlineStr">
+        <is>
+          <t>롯데건설</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Finalize Daily Work Report automation: RTK aggregation, OT consolidation, and Material name/spec mapping with manual overrides
</commit_message>
<xml_diff>
--- a/data/Material_Inventory.xlsx
+++ b/data/Material_Inventory.xlsx
@@ -22130,7 +22130,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W2"/>
+  <dimension ref="A1:W3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22252,10 +22252,10 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46137</v>
+        <v>46139</v>
       </c>
       <c r="B2" t="n">
-        <v>410</v>
+        <v>405</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -22263,36 +22263,36 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>-100</v>
+        <v>-50</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>K-1 PJT 현장 사용 (자동 차감)</t>
+          <t>K1 PJT 현장 사용 (자동 차감)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>부장 주진철, 부장 주동기</t>
+          <t>부장 주진철, 과장 유상훈, 계장 장승대</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>K-1 PJT</t>
+          <t>K1 PJT</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>스타렉스81루5100</t>
+          <t>스타렉스 0200</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>청결</t>
+          <t>out_exterior:양호|out_cleanliness:양호|out_cleaning:함|out_locking:잠금|in_exterior:양호|in_cleanliness:양호|in_cleaning:함|in_locking:잠금</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -22312,6 +22312,69 @@
       <c r="U2" t="inlineStr"/>
       <c r="V2" t="inlineStr"/>
       <c r="W2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="n">
+        <v>46139</v>
+      </c>
+      <c r="B3" t="n">
+        <v>406</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>-50</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>K1 PJT 현장 사용 (자동 차감)</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>부장 주진철, 과장 유상훈, 계장 장승대</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>K1 PJT</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>스타렉스 5100</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>out_exterior:양호|out_cleanliness:양호|out_cleaning:함|out_locking:잠금|in_exterior:양호|in_cleanliness:양호|in_cleaning:함|in_locking:잠금</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr"/>
+      <c r="R3" t="inlineStr"/>
+      <c r="S3" t="inlineStr"/>
+      <c r="T3" t="inlineStr"/>
+      <c r="U3" t="inlineStr"/>
+      <c r="V3" t="inlineStr"/>
+      <c r="W3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -22385,7 +22448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BX6"/>
+  <dimension ref="A1:CB5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22767,6 +22830,26 @@
       <c r="BX1" t="inlineStr">
         <is>
           <t>RTK_RTK총계</t>
+        </is>
+      </c>
+      <c r="BY1" t="inlineStr">
+        <is>
+          <t>검사품명</t>
+        </is>
+      </c>
+      <c r="BZ1" t="inlineStr">
+        <is>
+          <t>적용코드</t>
+        </is>
+      </c>
+      <c r="CA1" t="inlineStr">
+        <is>
+          <t>성적서번호</t>
+        </is>
+      </c>
+      <c r="CB1" t="inlineStr">
+        <is>
+          <t>검사자</t>
         </is>
       </c>
     </row>
@@ -22945,6 +23028,10 @@
       <c r="BX2" t="n">
         <v>0</v>
       </c>
+      <c r="BY2" t="inlineStr"/>
+      <c r="BZ2" t="inlineStr"/>
+      <c r="CA2" t="inlineStr"/>
+      <c r="CB2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr"/>
@@ -23121,34 +23208,38 @@
       <c r="BX3" t="n">
         <v>0</v>
       </c>
+      <c r="BY3" t="inlineStr"/>
+      <c r="BZ3" t="inlineStr"/>
+      <c r="CA3" t="inlineStr"/>
+      <c r="CB3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46137</v>
+        <v>46139</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>K-1 PJT</t>
+          <t>K1 PJT</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>410</v>
+        <v>405</v>
       </c>
       <c r="D4" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="E4" t="inlineStr"/>
       <c r="F4" s="1" t="n">
-        <v>46137.92250703704</v>
+        <v>46139.51755924769</v>
       </c>
       <c r="G4" t="n">
         <v>1</v>
       </c>
       <c r="H4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J4" t="n">
         <v>0</v>
@@ -23173,10 +23264,10 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="Q4" t="n">
-        <v>25500</v>
+        <v>25000</v>
       </c>
       <c r="R4" t="n">
         <v>0</v>
@@ -23185,7 +23276,7 @@
         <v>0</v>
       </c>
       <c r="T4" t="n">
-        <v>2550000</v>
+        <v>1250000</v>
       </c>
       <c r="U4" t="inlineStr">
         <is>
@@ -23197,32 +23288,44 @@
       </c>
       <c r="W4" t="inlineStr">
         <is>
-          <t>(휴일) 09:00~24:00</t>
+          <t>(주야간) 09:00~24:00</t>
         </is>
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>112,500</t>
+          <t>26,000</t>
         </is>
       </c>
       <c r="Y4" t="inlineStr">
         <is>
-          <t>부장 주동기</t>
+          <t>과장 유상훈</t>
         </is>
       </c>
       <c r="Z4" t="inlineStr">
         <is>
-          <t>(휴일) 09:00~24:00</t>
+          <t>(주야간) 09:00~24:00</t>
         </is>
       </c>
       <c r="AA4" t="inlineStr">
         <is>
-          <t>112,500</t>
-        </is>
-      </c>
-      <c r="AB4" t="inlineStr"/>
-      <c r="AC4" t="inlineStr"/>
-      <c r="AD4" t="inlineStr"/>
+          <t>26,000</t>
+        </is>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>계장 장승대</t>
+        </is>
+      </c>
+      <c r="AC4" t="inlineStr">
+        <is>
+          <t>(주야간) 09:00~24:00</t>
+        </is>
+      </c>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>26,000</t>
+        </is>
+      </c>
       <c r="AE4" t="inlineStr"/>
       <c r="AF4" t="inlineStr"/>
       <c r="AG4" t="inlineStr"/>
@@ -23270,17 +23373,13 @@
       </c>
       <c r="BH4" t="inlineStr">
         <is>
-          <t>스타렉스81루5100</t>
-        </is>
-      </c>
-      <c r="BI4" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
-      </c>
+          <t>스타렉스 0200</t>
+        </is>
+      </c>
+      <c r="BI4" t="inlineStr"/>
       <c r="BJ4" t="inlineStr">
         <is>
-          <t>청결</t>
+          <t>out_exterior:양호|out_cleanliness:양호|out_cleaning:함|out_locking:잠금|in_exterior:양호|in_cleanliness:양호|in_cleaning:함|in_locking:잠금</t>
         </is>
       </c>
       <c r="BK4" t="inlineStr"/>
@@ -23303,32 +23402,46 @@
       <c r="BV4" t="inlineStr"/>
       <c r="BW4" t="inlineStr"/>
       <c r="BX4" t="inlineStr"/>
+      <c r="BY4" t="inlineStr">
+        <is>
+          <t>PIPE</t>
+        </is>
+      </c>
+      <c r="BZ4" t="inlineStr">
+        <is>
+          <t>ASME B31.3</t>
+        </is>
+      </c>
+      <c r="CA4" t="inlineStr"/>
+      <c r="CB4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46120</v>
+        <v>46139</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>K-1 PJT</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr"/>
+          <t>K1 PJT</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>406</v>
+      </c>
       <c r="D5" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="E5" t="inlineStr"/>
       <c r="F5" s="1" t="n">
-        <v>46138.00012855324</v>
+        <v>46139.51798733796</v>
       </c>
       <c r="G5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H5" t="n">
         <v>0</v>
       </c>
       <c r="I5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J5" t="n">
         <v>0</v>
@@ -23349,14 +23462,14 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>PAUT 장비-OMNI2-103918</t>
+          <t>R-RAY</t>
         </is>
       </c>
       <c r="P5" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="Q5" t="n">
-        <v>18500</v>
+        <v>25000</v>
       </c>
       <c r="R5" t="n">
         <v>0</v>
@@ -23365,42 +23478,30 @@
         <v>0</v>
       </c>
       <c r="T5" t="n">
-        <v>1850000</v>
+        <v>1250000</v>
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>PAUT</t>
+          <t>RT</t>
         </is>
       </c>
       <c r="V5" t="n">
         <v>0</v>
       </c>
-      <c r="W5" t="inlineStr">
-        <is>
-          <t>(주야간) 09:00~24:00</t>
-        </is>
-      </c>
-      <c r="X5" t="inlineStr">
-        <is>
-          <t>26,000</t>
-        </is>
-      </c>
+      <c r="W5" t="inlineStr"/>
+      <c r="X5" t="inlineStr"/>
       <c r="Y5" t="inlineStr">
         <is>
-          <t>부장 주동기</t>
-        </is>
-      </c>
-      <c r="Z5" t="inlineStr">
-        <is>
-          <t>(주야간) 09:00~24:00</t>
-        </is>
-      </c>
-      <c r="AA5" t="inlineStr">
-        <is>
-          <t>26,000</t>
-        </is>
-      </c>
-      <c r="AB5" t="inlineStr"/>
+          <t>과장 유상훈</t>
+        </is>
+      </c>
+      <c r="Z5" t="inlineStr"/>
+      <c r="AA5" t="inlineStr"/>
+      <c r="AB5" t="inlineStr">
+        <is>
+          <t>계장 장승대</t>
+        </is>
+      </c>
       <c r="AC5" t="inlineStr"/>
       <c r="AD5" t="inlineStr"/>
       <c r="AE5" t="inlineStr"/>
@@ -23450,23 +23551,19 @@
       </c>
       <c r="BH5" t="inlineStr">
         <is>
-          <t>스타렉스81루5100</t>
-        </is>
-      </c>
-      <c r="BI5" t="inlineStr">
-        <is>
-          <t>80</t>
-        </is>
-      </c>
+          <t>스타렉스 5100</t>
+        </is>
+      </c>
+      <c r="BI5" t="inlineStr"/>
       <c r="BJ5" t="inlineStr">
         <is>
-          <t>청결</t>
+          <t>out_exterior:양호|out_cleanliness:양호|out_cleaning:함|out_locking:잠금|in_exterior:양호|in_cleanliness:양호|in_cleaning:함|in_locking:잠금</t>
         </is>
       </c>
       <c r="BK5" t="inlineStr"/>
       <c r="BL5" t="inlineStr"/>
       <c r="BM5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="BN5" t="inlineStr"/>
       <c r="BO5" t="inlineStr">
@@ -23483,188 +23580,18 @@
       <c r="BV5" t="inlineStr"/>
       <c r="BW5" t="inlineStr"/>
       <c r="BX5" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="1" t="n">
-        <v>46138</v>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>K-1 PJT</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>431</v>
-      </c>
-      <c r="D6" t="n">
-        <v>100</v>
-      </c>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" s="1" t="n">
-        <v>46138.46185664352</v>
-      </c>
-      <c r="G6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I6" t="n">
-        <v>0</v>
-      </c>
-      <c r="J6" t="n">
-        <v>0</v>
-      </c>
-      <c r="K6" t="n">
-        <v>0</v>
-      </c>
-      <c r="L6" t="n">
-        <v>0</v>
-      </c>
-      <c r="M6" t="n">
-        <v>0</v>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>부장 주진철</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>PAUT 장비-OMNI2-103918</t>
-        </is>
-      </c>
-      <c r="P6" t="n">
-        <v>100</v>
-      </c>
-      <c r="Q6" t="n">
-        <v>25500</v>
-      </c>
-      <c r="R6" t="n">
-        <v>0</v>
-      </c>
-      <c r="S6" t="n">
-        <v>0</v>
-      </c>
-      <c r="T6" t="n">
-        <v>2550000</v>
-      </c>
-      <c r="U6" t="inlineStr">
-        <is>
-          <t>PAUT</t>
-        </is>
-      </c>
-      <c r="V6" t="n">
-        <v>0</v>
-      </c>
-      <c r="W6" t="inlineStr">
-        <is>
-          <t>(휴일) 09:00~24:00</t>
-        </is>
-      </c>
-      <c r="X6" t="inlineStr">
-        <is>
-          <t>112,500</t>
-        </is>
-      </c>
-      <c r="Y6" t="inlineStr">
-        <is>
-          <t>부장 주동기</t>
-        </is>
-      </c>
-      <c r="Z6" t="inlineStr">
-        <is>
-          <t>09:00~18:00</t>
-        </is>
-      </c>
-      <c r="AA6" t="inlineStr">
-        <is>
-          <t>112,500</t>
-        </is>
-      </c>
-      <c r="AB6" t="inlineStr"/>
-      <c r="AC6" t="inlineStr"/>
-      <c r="AD6" t="inlineStr"/>
-      <c r="AE6" t="inlineStr"/>
-      <c r="AF6" t="inlineStr"/>
-      <c r="AG6" t="inlineStr"/>
-      <c r="AH6" t="inlineStr"/>
-      <c r="AI6" t="inlineStr"/>
-      <c r="AJ6" t="inlineStr"/>
-      <c r="AK6" t="inlineStr"/>
-      <c r="AL6" t="inlineStr"/>
-      <c r="AM6" t="inlineStr"/>
-      <c r="AN6" t="inlineStr"/>
-      <c r="AO6" t="inlineStr"/>
-      <c r="AP6" t="inlineStr"/>
-      <c r="AQ6" t="inlineStr"/>
-      <c r="AR6" t="inlineStr"/>
-      <c r="AS6" t="inlineStr"/>
-      <c r="AT6" t="inlineStr"/>
-      <c r="AU6" t="inlineStr"/>
-      <c r="AV6" t="inlineStr"/>
-      <c r="AW6" t="inlineStr"/>
-      <c r="AX6" t="inlineStr"/>
-      <c r="AY6" t="inlineStr"/>
-      <c r="AZ6" t="n">
-        <v>0</v>
-      </c>
-      <c r="BA6" t="n">
-        <v>0</v>
-      </c>
-      <c r="BB6" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC6" t="n">
-        <v>0</v>
-      </c>
-      <c r="BD6" t="n">
-        <v>0</v>
-      </c>
-      <c r="BE6" t="n">
-        <v>0</v>
-      </c>
-      <c r="BF6" t="n">
-        <v>0</v>
-      </c>
-      <c r="BG6" t="n">
-        <v>0</v>
-      </c>
-      <c r="BH6" t="inlineStr">
-        <is>
-          <t>스타렉스81루5100</t>
-        </is>
-      </c>
-      <c r="BI6" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
-      <c r="BJ6" t="inlineStr">
-        <is>
-          <t>청결</t>
-        </is>
-      </c>
-      <c r="BK6" t="inlineStr"/>
-      <c r="BL6" t="inlineStr"/>
-      <c r="BM6" t="n">
-        <v>0</v>
-      </c>
-      <c r="BN6" t="inlineStr"/>
-      <c r="BO6" t="inlineStr">
-        <is>
-          <t>롯데건설</t>
-        </is>
-      </c>
-      <c r="BP6" t="inlineStr"/>
-      <c r="BQ6" t="inlineStr"/>
-      <c r="BR6" t="inlineStr"/>
-      <c r="BS6" t="inlineStr"/>
-      <c r="BT6" t="inlineStr"/>
-      <c r="BU6" t="inlineStr"/>
-      <c r="BV6" t="inlineStr"/>
-      <c r="BW6" t="inlineStr"/>
-      <c r="BX6" t="inlineStr"/>
+      <c r="BY5" t="inlineStr">
+        <is>
+          <t>PIPE</t>
+        </is>
+      </c>
+      <c r="BZ5" t="inlineStr">
+        <is>
+          <t>ASME B31.3</t>
+        </is>
+      </c>
+      <c r="CA5" t="inlineStr"/>
+      <c r="CB5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
PAUT inventory logic refinement and data update
</commit_message>
<xml_diff>
--- a/data/Material_Inventory.xlsx
+++ b/data/Material_Inventory.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S430"/>
+  <dimension ref="A1:T433"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -519,6 +519,11 @@
       <c r="S1" t="inlineStr">
         <is>
           <t>Active</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>상태</t>
         </is>
       </c>
     </row>
@@ -574,6 +579,7 @@
       <c r="S2" t="n">
         <v>1</v>
       </c>
+      <c r="T2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -627,6 +633,7 @@
       <c r="S3" t="n">
         <v>1</v>
       </c>
+      <c r="T3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -680,6 +687,7 @@
       <c r="S4" t="n">
         <v>1</v>
       </c>
+      <c r="T4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -733,6 +741,7 @@
       <c r="S5" t="n">
         <v>1</v>
       </c>
+      <c r="T5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -786,6 +795,7 @@
       <c r="S6" t="n">
         <v>1</v>
       </c>
+      <c r="T6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -839,6 +849,7 @@
       <c r="S7" t="n">
         <v>1</v>
       </c>
+      <c r="T7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -892,6 +903,7 @@
       <c r="S8" t="n">
         <v>1</v>
       </c>
+      <c r="T8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -945,6 +957,7 @@
       <c r="S9" t="n">
         <v>1</v>
       </c>
+      <c r="T9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -998,6 +1011,7 @@
       <c r="S10" t="n">
         <v>1</v>
       </c>
+      <c r="T10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -1051,6 +1065,7 @@
       <c r="S11" t="n">
         <v>1</v>
       </c>
+      <c r="T11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -1104,6 +1119,7 @@
       <c r="S12" t="n">
         <v>1</v>
       </c>
+      <c r="T12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -1157,6 +1173,7 @@
       <c r="S13" t="n">
         <v>1</v>
       </c>
+      <c r="T13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -1210,6 +1227,7 @@
       <c r="S14" t="n">
         <v>1</v>
       </c>
+      <c r="T14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1263,6 +1281,7 @@
       <c r="S15" t="n">
         <v>1</v>
       </c>
+      <c r="T15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1316,6 +1335,7 @@
       <c r="S16" t="n">
         <v>1</v>
       </c>
+      <c r="T16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1369,6 +1389,7 @@
       <c r="S17" t="n">
         <v>1</v>
       </c>
+      <c r="T17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1422,6 +1443,7 @@
       <c r="S18" t="n">
         <v>1</v>
       </c>
+      <c r="T18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1475,6 +1497,7 @@
       <c r="S19" t="n">
         <v>1</v>
       </c>
+      <c r="T19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1528,6 +1551,7 @@
       <c r="S20" t="n">
         <v>1</v>
       </c>
+      <c r="T20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1581,6 +1605,7 @@
       <c r="S21" t="n">
         <v>1</v>
       </c>
+      <c r="T21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1634,6 +1659,7 @@
       <c r="S22" t="n">
         <v>1</v>
       </c>
+      <c r="T22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1687,6 +1713,7 @@
       <c r="S23" t="n">
         <v>1</v>
       </c>
+      <c r="T23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1740,6 +1767,7 @@
       <c r="S24" t="n">
         <v>1</v>
       </c>
+      <c r="T24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1793,6 +1821,7 @@
       <c r="S25" t="n">
         <v>1</v>
       </c>
+      <c r="T25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1846,6 +1875,7 @@
       <c r="S26" t="n">
         <v>1</v>
       </c>
+      <c r="T26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1899,6 +1929,7 @@
       <c r="S27" t="n">
         <v>1</v>
       </c>
+      <c r="T27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1952,6 +1983,7 @@
       <c r="S28" t="n">
         <v>1</v>
       </c>
+      <c r="T28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -2005,6 +2037,7 @@
       <c r="S29" t="n">
         <v>1</v>
       </c>
+      <c r="T29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -2058,6 +2091,7 @@
       <c r="S30" t="n">
         <v>1</v>
       </c>
+      <c r="T30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -2111,6 +2145,7 @@
       <c r="S31" t="n">
         <v>1</v>
       </c>
+      <c r="T31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -2164,6 +2199,7 @@
       <c r="S32" t="n">
         <v>1</v>
       </c>
+      <c r="T32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -2217,6 +2253,7 @@
       <c r="S33" t="n">
         <v>1</v>
       </c>
+      <c r="T33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -2270,6 +2307,7 @@
       <c r="S34" t="n">
         <v>1</v>
       </c>
+      <c r="T34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -2323,6 +2361,7 @@
       <c r="S35" t="n">
         <v>1</v>
       </c>
+      <c r="T35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -2376,6 +2415,7 @@
       <c r="S36" t="n">
         <v>1</v>
       </c>
+      <c r="T36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -2429,6 +2469,7 @@
       <c r="S37" t="n">
         <v>1</v>
       </c>
+      <c r="T37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -2482,6 +2523,7 @@
       <c r="S38" t="n">
         <v>1</v>
       </c>
+      <c r="T38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -2535,6 +2577,7 @@
       <c r="S39" t="n">
         <v>1</v>
       </c>
+      <c r="T39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -2588,6 +2631,7 @@
       <c r="S40" t="n">
         <v>1</v>
       </c>
+      <c r="T40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -2641,6 +2685,7 @@
       <c r="S41" t="n">
         <v>1</v>
       </c>
+      <c r="T41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -2694,6 +2739,7 @@
       <c r="S42" t="n">
         <v>1</v>
       </c>
+      <c r="T42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -2747,6 +2793,7 @@
       <c r="S43" t="n">
         <v>1</v>
       </c>
+      <c r="T43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -2800,6 +2847,7 @@
       <c r="S44" t="n">
         <v>1</v>
       </c>
+      <c r="T44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -2853,6 +2901,7 @@
       <c r="S45" t="n">
         <v>1</v>
       </c>
+      <c r="T45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -2906,6 +2955,7 @@
       <c r="S46" t="n">
         <v>1</v>
       </c>
+      <c r="T46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -2959,6 +3009,7 @@
       <c r="S47" t="n">
         <v>1</v>
       </c>
+      <c r="T47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -3008,6 +3059,7 @@
       <c r="S48" t="n">
         <v>1</v>
       </c>
+      <c r="T48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -3057,6 +3109,7 @@
       <c r="S49" t="n">
         <v>1</v>
       </c>
+      <c r="T49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -3106,6 +3159,7 @@
       <c r="S50" t="n">
         <v>1</v>
       </c>
+      <c r="T50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -3155,6 +3209,7 @@
       <c r="S51" t="n">
         <v>1</v>
       </c>
+      <c r="T51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -3204,6 +3259,7 @@
       <c r="S52" t="n">
         <v>1</v>
       </c>
+      <c r="T52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -3257,6 +3313,7 @@
       <c r="S53" t="n">
         <v>1</v>
       </c>
+      <c r="T53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -3310,6 +3367,7 @@
       <c r="S54" t="n">
         <v>1</v>
       </c>
+      <c r="T54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -3363,6 +3421,7 @@
       <c r="S55" t="n">
         <v>1</v>
       </c>
+      <c r="T55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -3416,6 +3475,7 @@
       <c r="S56" t="n">
         <v>1</v>
       </c>
+      <c r="T56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -3469,6 +3529,7 @@
       <c r="S57" t="n">
         <v>1</v>
       </c>
+      <c r="T57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -3522,6 +3583,7 @@
       <c r="S58" t="n">
         <v>1</v>
       </c>
+      <c r="T58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -3575,6 +3637,7 @@
       <c r="S59" t="n">
         <v>1</v>
       </c>
+      <c r="T59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -3628,6 +3691,7 @@
       <c r="S60" t="n">
         <v>1</v>
       </c>
+      <c r="T60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -3681,6 +3745,7 @@
       <c r="S61" t="n">
         <v>1</v>
       </c>
+      <c r="T61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -3734,6 +3799,7 @@
       <c r="S62" t="n">
         <v>1</v>
       </c>
+      <c r="T62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -3787,6 +3853,7 @@
       <c r="S63" t="n">
         <v>1</v>
       </c>
+      <c r="T63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -3840,6 +3907,7 @@
       <c r="S64" t="n">
         <v>1</v>
       </c>
+      <c r="T64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -3893,6 +3961,7 @@
       <c r="S65" t="n">
         <v>1</v>
       </c>
+      <c r="T65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -3946,6 +4015,7 @@
       <c r="S66" t="n">
         <v>1</v>
       </c>
+      <c r="T66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -3995,6 +4065,7 @@
       <c r="S67" t="n">
         <v>1</v>
       </c>
+      <c r="T67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -4044,6 +4115,7 @@
       <c r="S68" t="n">
         <v>1</v>
       </c>
+      <c r="T68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -4097,6 +4169,7 @@
       <c r="S69" t="n">
         <v>1</v>
       </c>
+      <c r="T69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -4150,6 +4223,7 @@
       <c r="S70" t="n">
         <v>1</v>
       </c>
+      <c r="T70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -4203,6 +4277,7 @@
       <c r="S71" t="n">
         <v>1</v>
       </c>
+      <c r="T71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -4256,6 +4331,7 @@
       <c r="S72" t="n">
         <v>1</v>
       </c>
+      <c r="T72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -4309,6 +4385,7 @@
       <c r="S73" t="n">
         <v>1</v>
       </c>
+      <c r="T73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -4362,6 +4439,7 @@
       <c r="S74" t="n">
         <v>1</v>
       </c>
+      <c r="T74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -4415,6 +4493,7 @@
       <c r="S75" t="n">
         <v>1</v>
       </c>
+      <c r="T75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -4468,6 +4547,7 @@
       <c r="S76" t="n">
         <v>1</v>
       </c>
+      <c r="T76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -4517,6 +4597,7 @@
       <c r="S77" t="n">
         <v>1</v>
       </c>
+      <c r="T77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -4570,6 +4651,7 @@
       <c r="S78" t="n">
         <v>1</v>
       </c>
+      <c r="T78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -4623,6 +4705,7 @@
       <c r="S79" t="n">
         <v>1</v>
       </c>
+      <c r="T79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -4676,6 +4759,7 @@
       <c r="S80" t="n">
         <v>1</v>
       </c>
+      <c r="T80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -4729,6 +4813,7 @@
       <c r="S81" t="n">
         <v>1</v>
       </c>
+      <c r="T81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -4782,6 +4867,7 @@
       <c r="S82" t="n">
         <v>1</v>
       </c>
+      <c r="T82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -4835,6 +4921,7 @@
       <c r="S83" t="n">
         <v>1</v>
       </c>
+      <c r="T83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -4888,6 +4975,7 @@
       <c r="S84" t="n">
         <v>1</v>
       </c>
+      <c r="T84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="n">
@@ -4941,6 +5029,7 @@
       <c r="S85" t="n">
         <v>1</v>
       </c>
+      <c r="T85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="n">
@@ -4990,6 +5079,7 @@
       <c r="S86" t="n">
         <v>1</v>
       </c>
+      <c r="T86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="n">
@@ -5039,6 +5129,7 @@
       <c r="S87" t="n">
         <v>1</v>
       </c>
+      <c r="T87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -5092,6 +5183,7 @@
       <c r="S88" t="n">
         <v>1</v>
       </c>
+      <c r="T88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -5145,6 +5237,7 @@
       <c r="S89" t="n">
         <v>1</v>
       </c>
+      <c r="T89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="n">
@@ -5198,6 +5291,7 @@
       <c r="S90" t="n">
         <v>1</v>
       </c>
+      <c r="T90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -5251,6 +5345,7 @@
       <c r="S91" t="n">
         <v>1</v>
       </c>
+      <c r="T91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -5300,6 +5395,7 @@
       <c r="S92" t="n">
         <v>1</v>
       </c>
+      <c r="T92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -5353,6 +5449,7 @@
       <c r="S93" t="n">
         <v>1</v>
       </c>
+      <c r="T93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -5402,6 +5499,7 @@
       <c r="S94" t="n">
         <v>1</v>
       </c>
+      <c r="T94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -5455,6 +5553,7 @@
       <c r="S95" t="n">
         <v>1</v>
       </c>
+      <c r="T95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -5508,6 +5607,7 @@
       <c r="S96" t="n">
         <v>1</v>
       </c>
+      <c r="T96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="n">
@@ -5553,6 +5653,7 @@
       <c r="S97" t="n">
         <v>1</v>
       </c>
+      <c r="T97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="n">
@@ -5598,6 +5699,7 @@
       <c r="S98" t="n">
         <v>1</v>
       </c>
+      <c r="T98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="n">
@@ -5643,6 +5745,7 @@
       <c r="S99" t="n">
         <v>1</v>
       </c>
+      <c r="T99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="n">
@@ -5688,6 +5791,7 @@
       <c r="S100" t="n">
         <v>1</v>
       </c>
+      <c r="T100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="n">
@@ -5733,6 +5837,7 @@
       <c r="S101" t="n">
         <v>1</v>
       </c>
+      <c r="T101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="n">
@@ -5778,6 +5883,7 @@
       <c r="S102" t="n">
         <v>1</v>
       </c>
+      <c r="T102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="n">
@@ -5823,6 +5929,7 @@
       <c r="S103" t="n">
         <v>1</v>
       </c>
+      <c r="T103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="n">
@@ -5868,6 +5975,7 @@
       <c r="S104" t="n">
         <v>1</v>
       </c>
+      <c r="T104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="n">
@@ -5913,6 +6021,7 @@
       <c r="S105" t="n">
         <v>1</v>
       </c>
+      <c r="T105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="n">
@@ -5958,6 +6067,7 @@
       <c r="S106" t="n">
         <v>1</v>
       </c>
+      <c r="T106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="n">
@@ -6003,6 +6113,7 @@
       <c r="S107" t="n">
         <v>1</v>
       </c>
+      <c r="T107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="n">
@@ -6048,6 +6159,7 @@
       <c r="S108" t="n">
         <v>1</v>
       </c>
+      <c r="T108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="n">
@@ -6093,6 +6205,7 @@
       <c r="S109" t="n">
         <v>1</v>
       </c>
+      <c r="T109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="n">
@@ -6138,6 +6251,7 @@
       <c r="S110" t="n">
         <v>1</v>
       </c>
+      <c r="T110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="n">
@@ -6183,6 +6297,7 @@
       <c r="S111" t="n">
         <v>1</v>
       </c>
+      <c r="T111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="n">
@@ -6228,6 +6343,7 @@
       <c r="S112" t="n">
         <v>1</v>
       </c>
+      <c r="T112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="n">
@@ -6273,6 +6389,7 @@
       <c r="S113" t="n">
         <v>1</v>
       </c>
+      <c r="T113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="n">
@@ -6318,6 +6435,7 @@
       <c r="S114" t="n">
         <v>1</v>
       </c>
+      <c r="T114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="n">
@@ -6363,6 +6481,7 @@
       <c r="S115" t="n">
         <v>1</v>
       </c>
+      <c r="T115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="n">
@@ -6408,6 +6527,7 @@
       <c r="S116" t="n">
         <v>1</v>
       </c>
+      <c r="T116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="n">
@@ -6453,6 +6573,7 @@
       <c r="S117" t="n">
         <v>1</v>
       </c>
+      <c r="T117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="n">
@@ -6498,6 +6619,7 @@
       <c r="S118" t="n">
         <v>1</v>
       </c>
+      <c r="T118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="n">
@@ -6543,6 +6665,7 @@
       <c r="S119" t="n">
         <v>1</v>
       </c>
+      <c r="T119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="n">
@@ -6588,6 +6711,7 @@
       <c r="S120" t="n">
         <v>1</v>
       </c>
+      <c r="T120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="n">
@@ -6633,6 +6757,7 @@
       <c r="S121" t="n">
         <v>1</v>
       </c>
+      <c r="T121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="n">
@@ -6678,6 +6803,7 @@
       <c r="S122" t="n">
         <v>1</v>
       </c>
+      <c r="T122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="n">
@@ -6723,6 +6849,7 @@
       <c r="S123" t="n">
         <v>1</v>
       </c>
+      <c r="T123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="n">
@@ -6768,6 +6895,7 @@
       <c r="S124" t="n">
         <v>1</v>
       </c>
+      <c r="T124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="n">
@@ -6813,6 +6941,7 @@
       <c r="S125" t="n">
         <v>1</v>
       </c>
+      <c r="T125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="n">
@@ -6858,6 +6987,7 @@
       <c r="S126" t="n">
         <v>1</v>
       </c>
+      <c r="T126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="n">
@@ -6903,6 +7033,7 @@
       <c r="S127" t="n">
         <v>1</v>
       </c>
+      <c r="T127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="n">
@@ -6948,6 +7079,7 @@
       <c r="S128" t="n">
         <v>1</v>
       </c>
+      <c r="T128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="n">
@@ -6993,6 +7125,7 @@
       <c r="S129" t="n">
         <v>1</v>
       </c>
+      <c r="T129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="n">
@@ -7038,6 +7171,7 @@
       <c r="S130" t="n">
         <v>1</v>
       </c>
+      <c r="T130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="n">
@@ -7083,6 +7217,7 @@
       <c r="S131" t="n">
         <v>1</v>
       </c>
+      <c r="T131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="n">
@@ -7128,6 +7263,7 @@
       <c r="S132" t="n">
         <v>1</v>
       </c>
+      <c r="T132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="n">
@@ -7173,6 +7309,7 @@
       <c r="S133" t="n">
         <v>1</v>
       </c>
+      <c r="T133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="n">
@@ -7218,6 +7355,7 @@
       <c r="S134" t="n">
         <v>1</v>
       </c>
+      <c r="T134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="n">
@@ -7263,6 +7401,7 @@
       <c r="S135" t="n">
         <v>1</v>
       </c>
+      <c r="T135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="n">
@@ -7308,6 +7447,7 @@
       <c r="S136" t="n">
         <v>1</v>
       </c>
+      <c r="T136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="n">
@@ -7353,6 +7493,7 @@
       <c r="S137" t="n">
         <v>1</v>
       </c>
+      <c r="T137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="n">
@@ -7398,6 +7539,7 @@
       <c r="S138" t="n">
         <v>1</v>
       </c>
+      <c r="T138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="n">
@@ -7443,6 +7585,7 @@
       <c r="S139" t="n">
         <v>1</v>
       </c>
+      <c r="T139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="n">
@@ -7488,6 +7631,7 @@
       <c r="S140" t="n">
         <v>1</v>
       </c>
+      <c r="T140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="n">
@@ -7533,6 +7677,7 @@
       <c r="S141" t="n">
         <v>1</v>
       </c>
+      <c r="T141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="n">
@@ -7578,6 +7723,7 @@
       <c r="S142" t="n">
         <v>1</v>
       </c>
+      <c r="T142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" t="n">
@@ -7623,6 +7769,7 @@
       <c r="S143" t="n">
         <v>1</v>
       </c>
+      <c r="T143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="n">
@@ -7668,6 +7815,7 @@
       <c r="S144" t="n">
         <v>1</v>
       </c>
+      <c r="T144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="n">
@@ -7713,6 +7861,7 @@
       <c r="S145" t="n">
         <v>1</v>
       </c>
+      <c r="T145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="n">
@@ -7758,6 +7907,7 @@
       <c r="S146" t="n">
         <v>1</v>
       </c>
+      <c r="T146" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" t="n">
@@ -7803,6 +7953,7 @@
       <c r="S147" t="n">
         <v>1</v>
       </c>
+      <c r="T147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" t="n">
@@ -7848,6 +7999,7 @@
       <c r="S148" t="n">
         <v>1</v>
       </c>
+      <c r="T148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" t="n">
@@ -7893,6 +8045,7 @@
       <c r="S149" t="n">
         <v>1</v>
       </c>
+      <c r="T149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" t="n">
@@ -7938,6 +8091,7 @@
       <c r="S150" t="n">
         <v>1</v>
       </c>
+      <c r="T150" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" t="n">
@@ -7983,6 +8137,7 @@
       <c r="S151" t="n">
         <v>1</v>
       </c>
+      <c r="T151" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" t="n">
@@ -8028,6 +8183,7 @@
       <c r="S152" t="n">
         <v>1</v>
       </c>
+      <c r="T152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" t="n">
@@ -8073,6 +8229,7 @@
       <c r="S153" t="n">
         <v>1</v>
       </c>
+      <c r="T153" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" t="n">
@@ -8118,6 +8275,7 @@
       <c r="S154" t="n">
         <v>1</v>
       </c>
+      <c r="T154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" t="n">
@@ -8163,6 +8321,7 @@
       <c r="S155" t="n">
         <v>1</v>
       </c>
+      <c r="T155" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" t="n">
@@ -8208,6 +8367,7 @@
       <c r="S156" t="n">
         <v>1</v>
       </c>
+      <c r="T156" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" t="n">
@@ -8253,6 +8413,7 @@
       <c r="S157" t="n">
         <v>1</v>
       </c>
+      <c r="T157" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" t="n">
@@ -8298,6 +8459,7 @@
       <c r="S158" t="n">
         <v>1</v>
       </c>
+      <c r="T158" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" t="n">
@@ -8343,6 +8505,7 @@
       <c r="S159" t="n">
         <v>1</v>
       </c>
+      <c r="T159" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" t="n">
@@ -8388,6 +8551,7 @@
       <c r="S160" t="n">
         <v>1</v>
       </c>
+      <c r="T160" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" t="n">
@@ -8433,6 +8597,7 @@
       <c r="S161" t="n">
         <v>1</v>
       </c>
+      <c r="T161" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" t="n">
@@ -8478,6 +8643,7 @@
       <c r="S162" t="n">
         <v>1</v>
       </c>
+      <c r="T162" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" t="n">
@@ -8523,6 +8689,7 @@
       <c r="S163" t="n">
         <v>1</v>
       </c>
+      <c r="T163" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" t="n">
@@ -8568,6 +8735,7 @@
       <c r="S164" t="n">
         <v>1</v>
       </c>
+      <c r="T164" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" t="n">
@@ -8613,6 +8781,7 @@
       <c r="S165" t="n">
         <v>1</v>
       </c>
+      <c r="T165" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" t="n">
@@ -8658,6 +8827,7 @@
       <c r="S166" t="n">
         <v>1</v>
       </c>
+      <c r="T166" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" t="n">
@@ -8703,6 +8873,7 @@
       <c r="S167" t="n">
         <v>1</v>
       </c>
+      <c r="T167" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" t="n">
@@ -8748,6 +8919,7 @@
       <c r="S168" t="n">
         <v>1</v>
       </c>
+      <c r="T168" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" t="n">
@@ -8793,6 +8965,7 @@
       <c r="S169" t="n">
         <v>1</v>
       </c>
+      <c r="T169" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" t="n">
@@ -8838,6 +9011,7 @@
       <c r="S170" t="n">
         <v>1</v>
       </c>
+      <c r="T170" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" t="n">
@@ -8883,6 +9057,7 @@
       <c r="S171" t="n">
         <v>1</v>
       </c>
+      <c r="T171" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" t="n">
@@ -8928,6 +9103,7 @@
       <c r="S172" t="n">
         <v>1</v>
       </c>
+      <c r="T172" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" t="n">
@@ -8973,6 +9149,7 @@
       <c r="S173" t="n">
         <v>1</v>
       </c>
+      <c r="T173" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" t="n">
@@ -9022,6 +9199,7 @@
       <c r="S174" t="n">
         <v>1</v>
       </c>
+      <c r="T174" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" t="n">
@@ -9075,6 +9253,7 @@
       <c r="S175" t="n">
         <v>1</v>
       </c>
+      <c r="T175" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" t="n">
@@ -9128,6 +9307,7 @@
       <c r="S176" t="n">
         <v>1</v>
       </c>
+      <c r="T176" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" t="n">
@@ -9173,6 +9353,7 @@
       <c r="S177" t="n">
         <v>1</v>
       </c>
+      <c r="T177" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" t="n">
@@ -9218,6 +9399,7 @@
       <c r="S178" t="n">
         <v>1</v>
       </c>
+      <c r="T178" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" t="n">
@@ -9263,6 +9445,7 @@
       <c r="S179" t="n">
         <v>1</v>
       </c>
+      <c r="T179" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" t="n">
@@ -9308,6 +9491,7 @@
       <c r="S180" t="n">
         <v>1</v>
       </c>
+      <c r="T180" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" t="n">
@@ -9353,6 +9537,7 @@
       <c r="S181" t="n">
         <v>1</v>
       </c>
+      <c r="T181" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" t="n">
@@ -9398,6 +9583,7 @@
       <c r="S182" t="n">
         <v>1</v>
       </c>
+      <c r="T182" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" t="n">
@@ -9443,6 +9629,7 @@
       <c r="S183" t="n">
         <v>1</v>
       </c>
+      <c r="T183" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" t="n">
@@ -9488,6 +9675,7 @@
       <c r="S184" t="n">
         <v>1</v>
       </c>
+      <c r="T184" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" t="n">
@@ -9533,6 +9721,7 @@
       <c r="S185" t="n">
         <v>1</v>
       </c>
+      <c r="T185" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" t="n">
@@ -9578,6 +9767,7 @@
       <c r="S186" t="n">
         <v>1</v>
       </c>
+      <c r="T186" t="inlineStr"/>
     </row>
     <row r="187">
       <c r="A187" t="n">
@@ -9623,6 +9813,7 @@
       <c r="S187" t="n">
         <v>1</v>
       </c>
+      <c r="T187" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" t="n">
@@ -9668,6 +9859,7 @@
       <c r="S188" t="n">
         <v>1</v>
       </c>
+      <c r="T188" t="inlineStr"/>
     </row>
     <row r="189">
       <c r="A189" t="n">
@@ -9713,6 +9905,7 @@
       <c r="S189" t="n">
         <v>1</v>
       </c>
+      <c r="T189" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" t="n">
@@ -9758,6 +9951,7 @@
       <c r="S190" t="n">
         <v>1</v>
       </c>
+      <c r="T190" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" t="n">
@@ -9803,6 +9997,7 @@
       <c r="S191" t="n">
         <v>1</v>
       </c>
+      <c r="T191" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" t="n">
@@ -9848,6 +10043,7 @@
       <c r="S192" t="n">
         <v>1</v>
       </c>
+      <c r="T192" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" t="n">
@@ -9893,6 +10089,7 @@
       <c r="S193" t="n">
         <v>1</v>
       </c>
+      <c r="T193" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" t="n">
@@ -9938,6 +10135,7 @@
       <c r="S194" t="n">
         <v>1</v>
       </c>
+      <c r="T194" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" t="n">
@@ -9983,6 +10181,7 @@
       <c r="S195" t="n">
         <v>1</v>
       </c>
+      <c r="T195" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" t="n">
@@ -10028,6 +10227,7 @@
       <c r="S196" t="n">
         <v>1</v>
       </c>
+      <c r="T196" t="inlineStr"/>
     </row>
     <row r="197">
       <c r="A197" t="n">
@@ -10073,6 +10273,7 @@
       <c r="S197" t="n">
         <v>1</v>
       </c>
+      <c r="T197" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" t="n">
@@ -10118,6 +10319,7 @@
       <c r="S198" t="n">
         <v>1</v>
       </c>
+      <c r="T198" t="inlineStr"/>
     </row>
     <row r="199">
       <c r="A199" t="n">
@@ -10163,6 +10365,7 @@
       <c r="S199" t="n">
         <v>1</v>
       </c>
+      <c r="T199" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" t="n">
@@ -10208,6 +10411,7 @@
       <c r="S200" t="n">
         <v>1</v>
       </c>
+      <c r="T200" t="inlineStr"/>
     </row>
     <row r="201">
       <c r="A201" t="n">
@@ -10253,6 +10457,7 @@
       <c r="S201" t="n">
         <v>1</v>
       </c>
+      <c r="T201" t="inlineStr"/>
     </row>
     <row r="202">
       <c r="A202" t="n">
@@ -10298,6 +10503,7 @@
       <c r="S202" t="n">
         <v>1</v>
       </c>
+      <c r="T202" t="inlineStr"/>
     </row>
     <row r="203">
       <c r="A203" t="n">
@@ -10343,6 +10549,7 @@
       <c r="S203" t="n">
         <v>1</v>
       </c>
+      <c r="T203" t="inlineStr"/>
     </row>
     <row r="204">
       <c r="A204" t="n">
@@ -10388,6 +10595,7 @@
       <c r="S204" t="n">
         <v>1</v>
       </c>
+      <c r="T204" t="inlineStr"/>
     </row>
     <row r="205">
       <c r="A205" t="n">
@@ -10433,6 +10641,7 @@
       <c r="S205" t="n">
         <v>1</v>
       </c>
+      <c r="T205" t="inlineStr"/>
     </row>
     <row r="206">
       <c r="A206" t="n">
@@ -10478,6 +10687,7 @@
       <c r="S206" t="n">
         <v>1</v>
       </c>
+      <c r="T206" t="inlineStr"/>
     </row>
     <row r="207">
       <c r="A207" t="n">
@@ -10523,6 +10733,7 @@
       <c r="S207" t="n">
         <v>1</v>
       </c>
+      <c r="T207" t="inlineStr"/>
     </row>
     <row r="208">
       <c r="A208" t="n">
@@ -10568,6 +10779,7 @@
       <c r="S208" t="n">
         <v>1</v>
       </c>
+      <c r="T208" t="inlineStr"/>
     </row>
     <row r="209">
       <c r="A209" t="n">
@@ -10613,6 +10825,7 @@
       <c r="S209" t="n">
         <v>1</v>
       </c>
+      <c r="T209" t="inlineStr"/>
     </row>
     <row r="210">
       <c r="A210" t="n">
@@ -10666,6 +10879,7 @@
       <c r="S210" t="n">
         <v>1</v>
       </c>
+      <c r="T210" t="inlineStr"/>
     </row>
     <row r="211">
       <c r="A211" t="n">
@@ -10719,6 +10933,7 @@
       <c r="S211" t="n">
         <v>1</v>
       </c>
+      <c r="T211" t="inlineStr"/>
     </row>
     <row r="212">
       <c r="A212" t="n">
@@ -10772,6 +10987,7 @@
       <c r="S212" t="n">
         <v>1</v>
       </c>
+      <c r="T212" t="inlineStr"/>
     </row>
     <row r="213">
       <c r="A213" t="n">
@@ -10825,6 +11041,7 @@
       <c r="S213" t="n">
         <v>1</v>
       </c>
+      <c r="T213" t="inlineStr"/>
     </row>
     <row r="214">
       <c r="A214" t="n">
@@ -10878,6 +11095,7 @@
       <c r="S214" t="n">
         <v>1</v>
       </c>
+      <c r="T214" t="inlineStr"/>
     </row>
     <row r="215">
       <c r="A215" t="n">
@@ -10931,6 +11149,7 @@
       <c r="S215" t="n">
         <v>1</v>
       </c>
+      <c r="T215" t="inlineStr"/>
     </row>
     <row r="216">
       <c r="A216" t="n">
@@ -10984,6 +11203,7 @@
       <c r="S216" t="n">
         <v>1</v>
       </c>
+      <c r="T216" t="inlineStr"/>
     </row>
     <row r="217">
       <c r="A217" t="n">
@@ -11037,6 +11257,7 @@
       <c r="S217" t="n">
         <v>1</v>
       </c>
+      <c r="T217" t="inlineStr"/>
     </row>
     <row r="218">
       <c r="A218" t="n">
@@ -11090,6 +11311,7 @@
       <c r="S218" t="n">
         <v>1</v>
       </c>
+      <c r="T218" t="inlineStr"/>
     </row>
     <row r="219">
       <c r="A219" t="n">
@@ -11143,6 +11365,7 @@
       <c r="S219" t="n">
         <v>1</v>
       </c>
+      <c r="T219" t="inlineStr"/>
     </row>
     <row r="220">
       <c r="A220" t="n">
@@ -11196,6 +11419,7 @@
       <c r="S220" t="n">
         <v>1</v>
       </c>
+      <c r="T220" t="inlineStr"/>
     </row>
     <row r="221">
       <c r="A221" t="n">
@@ -11249,6 +11473,7 @@
       <c r="S221" t="n">
         <v>1</v>
       </c>
+      <c r="T221" t="inlineStr"/>
     </row>
     <row r="222">
       <c r="A222" t="n">
@@ -11302,6 +11527,7 @@
       <c r="S222" t="n">
         <v>1</v>
       </c>
+      <c r="T222" t="inlineStr"/>
     </row>
     <row r="223">
       <c r="A223" t="n">
@@ -11355,6 +11581,7 @@
       <c r="S223" t="n">
         <v>1</v>
       </c>
+      <c r="T223" t="inlineStr"/>
     </row>
     <row r="224">
       <c r="A224" t="n">
@@ -11408,6 +11635,7 @@
       <c r="S224" t="n">
         <v>1</v>
       </c>
+      <c r="T224" t="inlineStr"/>
     </row>
     <row r="225">
       <c r="A225" t="n">
@@ -11461,6 +11689,7 @@
       <c r="S225" t="n">
         <v>1</v>
       </c>
+      <c r="T225" t="inlineStr"/>
     </row>
     <row r="226">
       <c r="A226" t="n">
@@ -11514,6 +11743,7 @@
       <c r="S226" t="n">
         <v>1</v>
       </c>
+      <c r="T226" t="inlineStr"/>
     </row>
     <row r="227">
       <c r="A227" t="n">
@@ -11567,6 +11797,7 @@
       <c r="S227" t="n">
         <v>1</v>
       </c>
+      <c r="T227" t="inlineStr"/>
     </row>
     <row r="228">
       <c r="A228" t="n">
@@ -11620,6 +11851,7 @@
       <c r="S228" t="n">
         <v>1</v>
       </c>
+      <c r="T228" t="inlineStr"/>
     </row>
     <row r="229">
       <c r="A229" t="n">
@@ -11669,6 +11901,7 @@
       <c r="S229" t="n">
         <v>1</v>
       </c>
+      <c r="T229" t="inlineStr"/>
     </row>
     <row r="230">
       <c r="A230" t="n">
@@ -11722,6 +11955,7 @@
       <c r="S230" t="n">
         <v>1</v>
       </c>
+      <c r="T230" t="inlineStr"/>
     </row>
     <row r="231">
       <c r="A231" t="n">
@@ -11775,6 +12009,7 @@
       <c r="S231" t="n">
         <v>1</v>
       </c>
+      <c r="T231" t="inlineStr"/>
     </row>
     <row r="232">
       <c r="A232" t="n">
@@ -11828,6 +12063,7 @@
       <c r="S232" t="n">
         <v>1</v>
       </c>
+      <c r="T232" t="inlineStr"/>
     </row>
     <row r="233">
       <c r="A233" t="n">
@@ -11881,6 +12117,7 @@
       <c r="S233" t="n">
         <v>1</v>
       </c>
+      <c r="T233" t="inlineStr"/>
     </row>
     <row r="234">
       <c r="A234" t="n">
@@ -11934,6 +12171,7 @@
       <c r="S234" t="n">
         <v>1</v>
       </c>
+      <c r="T234" t="inlineStr"/>
     </row>
     <row r="235">
       <c r="A235" t="n">
@@ -11987,6 +12225,7 @@
       <c r="S235" t="n">
         <v>1</v>
       </c>
+      <c r="T235" t="inlineStr"/>
     </row>
     <row r="236">
       <c r="A236" t="n">
@@ -12040,6 +12279,7 @@
       <c r="S236" t="n">
         <v>1</v>
       </c>
+      <c r="T236" t="inlineStr"/>
     </row>
     <row r="237">
       <c r="A237" t="n">
@@ -12093,6 +12333,7 @@
       <c r="S237" t="n">
         <v>1</v>
       </c>
+      <c r="T237" t="inlineStr"/>
     </row>
     <row r="238">
       <c r="A238" t="n">
@@ -12146,6 +12387,7 @@
       <c r="S238" t="n">
         <v>1</v>
       </c>
+      <c r="T238" t="inlineStr"/>
     </row>
     <row r="239">
       <c r="A239" t="n">
@@ -12199,6 +12441,7 @@
       <c r="S239" t="n">
         <v>1</v>
       </c>
+      <c r="T239" t="inlineStr"/>
     </row>
     <row r="240">
       <c r="A240" t="n">
@@ -12252,6 +12495,7 @@
       <c r="S240" t="n">
         <v>1</v>
       </c>
+      <c r="T240" t="inlineStr"/>
     </row>
     <row r="241">
       <c r="A241" t="n">
@@ -12305,6 +12549,7 @@
       <c r="S241" t="n">
         <v>1</v>
       </c>
+      <c r="T241" t="inlineStr"/>
     </row>
     <row r="242">
       <c r="A242" t="n">
@@ -12358,6 +12603,7 @@
       <c r="S242" t="n">
         <v>1</v>
       </c>
+      <c r="T242" t="inlineStr"/>
     </row>
     <row r="243">
       <c r="A243" t="n">
@@ -12411,6 +12657,7 @@
       <c r="S243" t="n">
         <v>1</v>
       </c>
+      <c r="T243" t="inlineStr"/>
     </row>
     <row r="244">
       <c r="A244" t="n">
@@ -12464,6 +12711,7 @@
       <c r="S244" t="n">
         <v>1</v>
       </c>
+      <c r="T244" t="inlineStr"/>
     </row>
     <row r="245">
       <c r="A245" t="n">
@@ -12513,6 +12761,7 @@
       <c r="S245" t="n">
         <v>1</v>
       </c>
+      <c r="T245" t="inlineStr"/>
     </row>
     <row r="246">
       <c r="A246" t="n">
@@ -12562,6 +12811,7 @@
       <c r="S246" t="n">
         <v>1</v>
       </c>
+      <c r="T246" t="inlineStr"/>
     </row>
     <row r="247">
       <c r="A247" t="n">
@@ -12611,6 +12861,7 @@
       <c r="S247" t="n">
         <v>1</v>
       </c>
+      <c r="T247" t="inlineStr"/>
     </row>
     <row r="248">
       <c r="A248" t="n">
@@ -12664,6 +12915,7 @@
       <c r="S248" t="n">
         <v>1</v>
       </c>
+      <c r="T248" t="inlineStr"/>
     </row>
     <row r="249">
       <c r="A249" t="n">
@@ -12717,6 +12969,7 @@
       <c r="S249" t="n">
         <v>1</v>
       </c>
+      <c r="T249" t="inlineStr"/>
     </row>
     <row r="250">
       <c r="A250" t="n">
@@ -12766,6 +13019,7 @@
       <c r="S250" t="n">
         <v>1</v>
       </c>
+      <c r="T250" t="inlineStr"/>
     </row>
     <row r="251">
       <c r="A251" t="n">
@@ -12819,6 +13073,7 @@
       <c r="S251" t="n">
         <v>1</v>
       </c>
+      <c r="T251" t="inlineStr"/>
     </row>
     <row r="252">
       <c r="A252" t="n">
@@ -12868,6 +13123,7 @@
       <c r="S252" t="n">
         <v>1</v>
       </c>
+      <c r="T252" t="inlineStr"/>
     </row>
     <row r="253">
       <c r="A253" t="n">
@@ -12917,6 +13173,7 @@
       <c r="S253" t="n">
         <v>1</v>
       </c>
+      <c r="T253" t="inlineStr"/>
     </row>
     <row r="254">
       <c r="A254" t="n">
@@ -12970,6 +13227,7 @@
       <c r="S254" t="n">
         <v>1</v>
       </c>
+      <c r="T254" t="inlineStr"/>
     </row>
     <row r="255">
       <c r="A255" t="n">
@@ -13023,6 +13281,7 @@
       <c r="S255" t="n">
         <v>1</v>
       </c>
+      <c r="T255" t="inlineStr"/>
     </row>
     <row r="256">
       <c r="A256" t="n">
@@ -13076,6 +13335,7 @@
       <c r="S256" t="n">
         <v>1</v>
       </c>
+      <c r="T256" t="inlineStr"/>
     </row>
     <row r="257">
       <c r="A257" t="n">
@@ -13129,6 +13389,7 @@
       <c r="S257" t="n">
         <v>1</v>
       </c>
+      <c r="T257" t="inlineStr"/>
     </row>
     <row r="258">
       <c r="A258" t="n">
@@ -13182,6 +13443,7 @@
       <c r="S258" t="n">
         <v>1</v>
       </c>
+      <c r="T258" t="inlineStr"/>
     </row>
     <row r="259">
       <c r="A259" t="n">
@@ -13235,6 +13497,7 @@
       <c r="S259" t="n">
         <v>1</v>
       </c>
+      <c r="T259" t="inlineStr"/>
     </row>
     <row r="260">
       <c r="A260" t="n">
@@ -13288,6 +13551,7 @@
       <c r="S260" t="n">
         <v>1</v>
       </c>
+      <c r="T260" t="inlineStr"/>
     </row>
     <row r="261">
       <c r="A261" t="n">
@@ -13337,6 +13601,7 @@
       <c r="S261" t="n">
         <v>1</v>
       </c>
+      <c r="T261" t="inlineStr"/>
     </row>
     <row r="262">
       <c r="A262" t="n">
@@ -13390,6 +13655,7 @@
       <c r="S262" t="n">
         <v>1</v>
       </c>
+      <c r="T262" t="inlineStr"/>
     </row>
     <row r="263">
       <c r="A263" t="n">
@@ -13443,6 +13709,7 @@
       <c r="S263" t="n">
         <v>1</v>
       </c>
+      <c r="T263" t="inlineStr"/>
     </row>
     <row r="264">
       <c r="A264" t="n">
@@ -13496,6 +13763,7 @@
       <c r="S264" t="n">
         <v>1</v>
       </c>
+      <c r="T264" t="inlineStr"/>
     </row>
     <row r="265">
       <c r="A265" t="n">
@@ -13549,6 +13817,7 @@
       <c r="S265" t="n">
         <v>1</v>
       </c>
+      <c r="T265" t="inlineStr"/>
     </row>
     <row r="266">
       <c r="A266" t="n">
@@ -13602,6 +13871,7 @@
       <c r="S266" t="n">
         <v>1</v>
       </c>
+      <c r="T266" t="inlineStr"/>
     </row>
     <row r="267">
       <c r="A267" t="n">
@@ -13655,6 +13925,7 @@
       <c r="S267" t="n">
         <v>1</v>
       </c>
+      <c r="T267" t="inlineStr"/>
     </row>
     <row r="268">
       <c r="A268" t="n">
@@ -13708,6 +13979,7 @@
       <c r="S268" t="n">
         <v>1</v>
       </c>
+      <c r="T268" t="inlineStr"/>
     </row>
     <row r="269">
       <c r="A269" t="n">
@@ -13761,6 +14033,7 @@
       <c r="S269" t="n">
         <v>1</v>
       </c>
+      <c r="T269" t="inlineStr"/>
     </row>
     <row r="270">
       <c r="A270" t="n">
@@ -13814,6 +14087,7 @@
       <c r="S270" t="n">
         <v>1</v>
       </c>
+      <c r="T270" t="inlineStr"/>
     </row>
     <row r="271">
       <c r="A271" t="n">
@@ -13867,6 +14141,7 @@
       <c r="S271" t="n">
         <v>1</v>
       </c>
+      <c r="T271" t="inlineStr"/>
     </row>
     <row r="272">
       <c r="A272" t="n">
@@ -13920,6 +14195,7 @@
       <c r="S272" t="n">
         <v>1</v>
       </c>
+      <c r="T272" t="inlineStr"/>
     </row>
     <row r="273">
       <c r="A273" t="n">
@@ -13973,6 +14249,7 @@
       <c r="S273" t="n">
         <v>1</v>
       </c>
+      <c r="T273" t="inlineStr"/>
     </row>
     <row r="274">
       <c r="A274" t="n">
@@ -14026,6 +14303,7 @@
       <c r="S274" t="n">
         <v>1</v>
       </c>
+      <c r="T274" t="inlineStr"/>
     </row>
     <row r="275">
       <c r="A275" t="n">
@@ -14079,6 +14357,7 @@
       <c r="S275" t="n">
         <v>1</v>
       </c>
+      <c r="T275" t="inlineStr"/>
     </row>
     <row r="276">
       <c r="A276" t="n">
@@ -14132,6 +14411,7 @@
       <c r="S276" t="n">
         <v>1</v>
       </c>
+      <c r="T276" t="inlineStr"/>
     </row>
     <row r="277">
       <c r="A277" t="n">
@@ -14185,6 +14465,7 @@
       <c r="S277" t="n">
         <v>1</v>
       </c>
+      <c r="T277" t="inlineStr"/>
     </row>
     <row r="278">
       <c r="A278" t="n">
@@ -14238,6 +14519,7 @@
       <c r="S278" t="n">
         <v>1</v>
       </c>
+      <c r="T278" t="inlineStr"/>
     </row>
     <row r="279">
       <c r="A279" t="n">
@@ -14291,6 +14573,7 @@
       <c r="S279" t="n">
         <v>1</v>
       </c>
+      <c r="T279" t="inlineStr"/>
     </row>
     <row r="280">
       <c r="A280" t="n">
@@ -14344,6 +14627,7 @@
       <c r="S280" t="n">
         <v>1</v>
       </c>
+      <c r="T280" t="inlineStr"/>
     </row>
     <row r="281">
       <c r="A281" t="n">
@@ -14397,6 +14681,7 @@
       <c r="S281" t="n">
         <v>1</v>
       </c>
+      <c r="T281" t="inlineStr"/>
     </row>
     <row r="282">
       <c r="A282" t="n">
@@ -14450,6 +14735,7 @@
       <c r="S282" t="n">
         <v>1</v>
       </c>
+      <c r="T282" t="inlineStr"/>
     </row>
     <row r="283">
       <c r="A283" t="n">
@@ -14503,6 +14789,7 @@
       <c r="S283" t="n">
         <v>1</v>
       </c>
+      <c r="T283" t="inlineStr"/>
     </row>
     <row r="284">
       <c r="A284" t="n">
@@ -14556,6 +14843,7 @@
       <c r="S284" t="n">
         <v>1</v>
       </c>
+      <c r="T284" t="inlineStr"/>
     </row>
     <row r="285">
       <c r="A285" t="n">
@@ -14609,6 +14897,7 @@
       <c r="S285" t="n">
         <v>1</v>
       </c>
+      <c r="T285" t="inlineStr"/>
     </row>
     <row r="286">
       <c r="A286" t="n">
@@ -14662,6 +14951,7 @@
       <c r="S286" t="n">
         <v>1</v>
       </c>
+      <c r="T286" t="inlineStr"/>
     </row>
     <row r="287">
       <c r="A287" t="n">
@@ -14715,6 +15005,7 @@
       <c r="S287" t="n">
         <v>1</v>
       </c>
+      <c r="T287" t="inlineStr"/>
     </row>
     <row r="288">
       <c r="A288" t="n">
@@ -14768,6 +15059,7 @@
       <c r="S288" t="n">
         <v>1</v>
       </c>
+      <c r="T288" t="inlineStr"/>
     </row>
     <row r="289">
       <c r="A289" t="n">
@@ -14821,6 +15113,7 @@
       <c r="S289" t="n">
         <v>1</v>
       </c>
+      <c r="T289" t="inlineStr"/>
     </row>
     <row r="290">
       <c r="A290" t="n">
@@ -14874,6 +15167,7 @@
       <c r="S290" t="n">
         <v>1</v>
       </c>
+      <c r="T290" t="inlineStr"/>
     </row>
     <row r="291">
       <c r="A291" t="n">
@@ -14927,6 +15221,7 @@
       <c r="S291" t="n">
         <v>1</v>
       </c>
+      <c r="T291" t="inlineStr"/>
     </row>
     <row r="292">
       <c r="A292" t="n">
@@ -14980,6 +15275,7 @@
       <c r="S292" t="n">
         <v>1</v>
       </c>
+      <c r="T292" t="inlineStr"/>
     </row>
     <row r="293">
       <c r="A293" t="n">
@@ -15033,6 +15329,7 @@
       <c r="S293" t="n">
         <v>1</v>
       </c>
+      <c r="T293" t="inlineStr"/>
     </row>
     <row r="294">
       <c r="A294" t="n">
@@ -15086,6 +15383,7 @@
       <c r="S294" t="n">
         <v>1</v>
       </c>
+      <c r="T294" t="inlineStr"/>
     </row>
     <row r="295">
       <c r="A295" t="n">
@@ -15139,6 +15437,7 @@
       <c r="S295" t="n">
         <v>1</v>
       </c>
+      <c r="T295" t="inlineStr"/>
     </row>
     <row r="296">
       <c r="A296" t="n">
@@ -15192,6 +15491,7 @@
       <c r="S296" t="n">
         <v>1</v>
       </c>
+      <c r="T296" t="inlineStr"/>
     </row>
     <row r="297">
       <c r="A297" t="n">
@@ -15245,6 +15545,7 @@
       <c r="S297" t="n">
         <v>1</v>
       </c>
+      <c r="T297" t="inlineStr"/>
     </row>
     <row r="298">
       <c r="A298" t="n">
@@ -15298,6 +15599,7 @@
       <c r="S298" t="n">
         <v>1</v>
       </c>
+      <c r="T298" t="inlineStr"/>
     </row>
     <row r="299">
       <c r="A299" t="n">
@@ -15351,6 +15653,7 @@
       <c r="S299" t="n">
         <v>1</v>
       </c>
+      <c r="T299" t="inlineStr"/>
     </row>
     <row r="300">
       <c r="A300" t="n">
@@ -15404,6 +15707,7 @@
       <c r="S300" t="n">
         <v>1</v>
       </c>
+      <c r="T300" t="inlineStr"/>
     </row>
     <row r="301">
       <c r="A301" t="n">
@@ -15457,6 +15761,7 @@
       <c r="S301" t="n">
         <v>1</v>
       </c>
+      <c r="T301" t="inlineStr"/>
     </row>
     <row r="302">
       <c r="A302" t="n">
@@ -15510,6 +15815,7 @@
       <c r="S302" t="n">
         <v>1</v>
       </c>
+      <c r="T302" t="inlineStr"/>
     </row>
     <row r="303">
       <c r="A303" t="n">
@@ -15563,6 +15869,7 @@
       <c r="S303" t="n">
         <v>1</v>
       </c>
+      <c r="T303" t="inlineStr"/>
     </row>
     <row r="304">
       <c r="A304" t="n">
@@ -15616,6 +15923,7 @@
       <c r="S304" t="n">
         <v>1</v>
       </c>
+      <c r="T304" t="inlineStr"/>
     </row>
     <row r="305">
       <c r="A305" t="n">
@@ -15669,6 +15977,7 @@
       <c r="S305" t="n">
         <v>1</v>
       </c>
+      <c r="T305" t="inlineStr"/>
     </row>
     <row r="306">
       <c r="A306" t="n">
@@ -15722,6 +16031,7 @@
       <c r="S306" t="n">
         <v>1</v>
       </c>
+      <c r="T306" t="inlineStr"/>
     </row>
     <row r="307">
       <c r="A307" t="n">
@@ -15775,6 +16085,7 @@
       <c r="S307" t="n">
         <v>1</v>
       </c>
+      <c r="T307" t="inlineStr"/>
     </row>
     <row r="308">
       <c r="A308" t="n">
@@ -15828,6 +16139,7 @@
       <c r="S308" t="n">
         <v>1</v>
       </c>
+      <c r="T308" t="inlineStr"/>
     </row>
     <row r="309">
       <c r="A309" t="n">
@@ -15881,6 +16193,7 @@
       <c r="S309" t="n">
         <v>1</v>
       </c>
+      <c r="T309" t="inlineStr"/>
     </row>
     <row r="310">
       <c r="A310" t="n">
@@ -15934,6 +16247,7 @@
       <c r="S310" t="n">
         <v>1</v>
       </c>
+      <c r="T310" t="inlineStr"/>
     </row>
     <row r="311">
       <c r="A311" t="n">
@@ -15987,6 +16301,7 @@
       <c r="S311" t="n">
         <v>1</v>
       </c>
+      <c r="T311" t="inlineStr"/>
     </row>
     <row r="312">
       <c r="A312" t="n">
@@ -16040,6 +16355,7 @@
       <c r="S312" t="n">
         <v>1</v>
       </c>
+      <c r="T312" t="inlineStr"/>
     </row>
     <row r="313">
       <c r="A313" t="n">
@@ -16093,6 +16409,7 @@
       <c r="S313" t="n">
         <v>1</v>
       </c>
+      <c r="T313" t="inlineStr"/>
     </row>
     <row r="314">
       <c r="A314" t="n">
@@ -16146,6 +16463,7 @@
       <c r="S314" t="n">
         <v>1</v>
       </c>
+      <c r="T314" t="inlineStr"/>
     </row>
     <row r="315">
       <c r="A315" t="n">
@@ -16199,6 +16517,7 @@
       <c r="S315" t="n">
         <v>1</v>
       </c>
+      <c r="T315" t="inlineStr"/>
     </row>
     <row r="316">
       <c r="A316" t="n">
@@ -16252,6 +16571,7 @@
       <c r="S316" t="n">
         <v>1</v>
       </c>
+      <c r="T316" t="inlineStr"/>
     </row>
     <row r="317">
       <c r="A317" t="n">
@@ -16305,6 +16625,7 @@
       <c r="S317" t="n">
         <v>1</v>
       </c>
+      <c r="T317" t="inlineStr"/>
     </row>
     <row r="318">
       <c r="A318" t="n">
@@ -16358,6 +16679,7 @@
       <c r="S318" t="n">
         <v>1</v>
       </c>
+      <c r="T318" t="inlineStr"/>
     </row>
     <row r="319">
       <c r="A319" t="n">
@@ -16411,6 +16733,7 @@
       <c r="S319" t="n">
         <v>1</v>
       </c>
+      <c r="T319" t="inlineStr"/>
     </row>
     <row r="320">
       <c r="A320" t="n">
@@ -16464,6 +16787,7 @@
       <c r="S320" t="n">
         <v>1</v>
       </c>
+      <c r="T320" t="inlineStr"/>
     </row>
     <row r="321">
       <c r="A321" t="n">
@@ -16517,6 +16841,7 @@
       <c r="S321" t="n">
         <v>1</v>
       </c>
+      <c r="T321" t="inlineStr"/>
     </row>
     <row r="322">
       <c r="A322" t="n">
@@ -16570,6 +16895,7 @@
       <c r="S322" t="n">
         <v>1</v>
       </c>
+      <c r="T322" t="inlineStr"/>
     </row>
     <row r="323">
       <c r="A323" t="n">
@@ -16623,6 +16949,7 @@
       <c r="S323" t="n">
         <v>1</v>
       </c>
+      <c r="T323" t="inlineStr"/>
     </row>
     <row r="324">
       <c r="A324" t="n">
@@ -16676,6 +17003,7 @@
       <c r="S324" t="n">
         <v>1</v>
       </c>
+      <c r="T324" t="inlineStr"/>
     </row>
     <row r="325">
       <c r="A325" t="n">
@@ -16729,6 +17057,7 @@
       <c r="S325" t="n">
         <v>1</v>
       </c>
+      <c r="T325" t="inlineStr"/>
     </row>
     <row r="326">
       <c r="A326" t="n">
@@ -16782,6 +17111,7 @@
       <c r="S326" t="n">
         <v>1</v>
       </c>
+      <c r="T326" t="inlineStr"/>
     </row>
     <row r="327">
       <c r="A327" t="n">
@@ -16835,6 +17165,7 @@
       <c r="S327" t="n">
         <v>1</v>
       </c>
+      <c r="T327" t="inlineStr"/>
     </row>
     <row r="328">
       <c r="A328" t="n">
@@ -16888,6 +17219,7 @@
       <c r="S328" t="n">
         <v>1</v>
       </c>
+      <c r="T328" t="inlineStr"/>
     </row>
     <row r="329">
       <c r="A329" t="n">
@@ -16941,6 +17273,7 @@
       <c r="S329" t="n">
         <v>1</v>
       </c>
+      <c r="T329" t="inlineStr"/>
     </row>
     <row r="330">
       <c r="A330" t="n">
@@ -16994,6 +17327,7 @@
       <c r="S330" t="n">
         <v>1</v>
       </c>
+      <c r="T330" t="inlineStr"/>
     </row>
     <row r="331">
       <c r="A331" t="n">
@@ -17047,6 +17381,7 @@
       <c r="S331" t="n">
         <v>1</v>
       </c>
+      <c r="T331" t="inlineStr"/>
     </row>
     <row r="332">
       <c r="A332" t="n">
@@ -17100,6 +17435,7 @@
       <c r="S332" t="n">
         <v>1</v>
       </c>
+      <c r="T332" t="inlineStr"/>
     </row>
     <row r="333">
       <c r="A333" t="n">
@@ -17153,6 +17489,7 @@
       <c r="S333" t="n">
         <v>1</v>
       </c>
+      <c r="T333" t="inlineStr"/>
     </row>
     <row r="334">
       <c r="A334" t="n">
@@ -17206,6 +17543,7 @@
       <c r="S334" t="n">
         <v>1</v>
       </c>
+      <c r="T334" t="inlineStr"/>
     </row>
     <row r="335">
       <c r="A335" t="n">
@@ -17259,6 +17597,7 @@
       <c r="S335" t="n">
         <v>1</v>
       </c>
+      <c r="T335" t="inlineStr"/>
     </row>
     <row r="336">
       <c r="A336" t="n">
@@ -17312,6 +17651,7 @@
       <c r="S336" t="n">
         <v>1</v>
       </c>
+      <c r="T336" t="inlineStr"/>
     </row>
     <row r="337">
       <c r="A337" t="n">
@@ -17365,6 +17705,7 @@
       <c r="S337" t="n">
         <v>1</v>
       </c>
+      <c r="T337" t="inlineStr"/>
     </row>
     <row r="338">
       <c r="A338" t="n">
@@ -17418,6 +17759,7 @@
       <c r="S338" t="n">
         <v>1</v>
       </c>
+      <c r="T338" t="inlineStr"/>
     </row>
     <row r="339">
       <c r="A339" t="n">
@@ -17471,6 +17813,7 @@
       <c r="S339" t="n">
         <v>1</v>
       </c>
+      <c r="T339" t="inlineStr"/>
     </row>
     <row r="340">
       <c r="A340" t="n">
@@ -17524,6 +17867,7 @@
       <c r="S340" t="n">
         <v>1</v>
       </c>
+      <c r="T340" t="inlineStr"/>
     </row>
     <row r="341">
       <c r="A341" t="n">
@@ -17577,6 +17921,7 @@
       <c r="S341" t="n">
         <v>1</v>
       </c>
+      <c r="T341" t="inlineStr"/>
     </row>
     <row r="342">
       <c r="A342" t="n">
@@ -17630,6 +17975,7 @@
       <c r="S342" t="n">
         <v>1</v>
       </c>
+      <c r="T342" t="inlineStr"/>
     </row>
     <row r="343">
       <c r="A343" t="n">
@@ -17683,6 +18029,7 @@
       <c r="S343" t="n">
         <v>1</v>
       </c>
+      <c r="T343" t="inlineStr"/>
     </row>
     <row r="344">
       <c r="A344" t="n">
@@ -17736,6 +18083,7 @@
       <c r="S344" t="n">
         <v>1</v>
       </c>
+      <c r="T344" t="inlineStr"/>
     </row>
     <row r="345">
       <c r="A345" t="n">
@@ -17789,6 +18137,7 @@
       <c r="S345" t="n">
         <v>1</v>
       </c>
+      <c r="T345" t="inlineStr"/>
     </row>
     <row r="346">
       <c r="A346" t="n">
@@ -17842,6 +18191,7 @@
       <c r="S346" t="n">
         <v>1</v>
       </c>
+      <c r="T346" t="inlineStr"/>
     </row>
     <row r="347">
       <c r="A347" t="n">
@@ -17895,6 +18245,7 @@
       <c r="S347" t="n">
         <v>1</v>
       </c>
+      <c r="T347" t="inlineStr"/>
     </row>
     <row r="348">
       <c r="A348" t="n">
@@ -17948,6 +18299,7 @@
       <c r="S348" t="n">
         <v>1</v>
       </c>
+      <c r="T348" t="inlineStr"/>
     </row>
     <row r="349">
       <c r="A349" t="n">
@@ -18001,6 +18353,7 @@
       <c r="S349" t="n">
         <v>1</v>
       </c>
+      <c r="T349" t="inlineStr"/>
     </row>
     <row r="350">
       <c r="A350" t="n">
@@ -18054,6 +18407,7 @@
       <c r="S350" t="n">
         <v>1</v>
       </c>
+      <c r="T350" t="inlineStr"/>
     </row>
     <row r="351">
       <c r="A351" t="n">
@@ -18107,6 +18461,7 @@
       <c r="S351" t="n">
         <v>1</v>
       </c>
+      <c r="T351" t="inlineStr"/>
     </row>
     <row r="352">
       <c r="A352" t="n">
@@ -18160,6 +18515,7 @@
       <c r="S352" t="n">
         <v>1</v>
       </c>
+      <c r="T352" t="inlineStr"/>
     </row>
     <row r="353">
       <c r="A353" t="n">
@@ -18213,6 +18569,7 @@
       <c r="S353" t="n">
         <v>1</v>
       </c>
+      <c r="T353" t="inlineStr"/>
     </row>
     <row r="354">
       <c r="A354" t="n">
@@ -18266,6 +18623,7 @@
       <c r="S354" t="n">
         <v>1</v>
       </c>
+      <c r="T354" t="inlineStr"/>
     </row>
     <row r="355">
       <c r="A355" t="n">
@@ -18319,6 +18677,7 @@
       <c r="S355" t="n">
         <v>1</v>
       </c>
+      <c r="T355" t="inlineStr"/>
     </row>
     <row r="356">
       <c r="A356" t="n">
@@ -18372,6 +18731,7 @@
       <c r="S356" t="n">
         <v>1</v>
       </c>
+      <c r="T356" t="inlineStr"/>
     </row>
     <row r="357">
       <c r="A357" t="n">
@@ -18421,6 +18781,7 @@
       <c r="S357" t="n">
         <v>1</v>
       </c>
+      <c r="T357" t="inlineStr"/>
     </row>
     <row r="358">
       <c r="A358" t="n">
@@ -18474,6 +18835,7 @@
       <c r="S358" t="n">
         <v>1</v>
       </c>
+      <c r="T358" t="inlineStr"/>
     </row>
     <row r="359">
       <c r="A359" t="n">
@@ -18523,6 +18885,7 @@
       <c r="S359" t="n">
         <v>1</v>
       </c>
+      <c r="T359" t="inlineStr"/>
     </row>
     <row r="360">
       <c r="A360" t="n">
@@ -18572,6 +18935,7 @@
       <c r="S360" t="n">
         <v>1</v>
       </c>
+      <c r="T360" t="inlineStr"/>
     </row>
     <row r="361">
       <c r="A361" t="n">
@@ -18621,6 +18985,7 @@
       <c r="S361" t="n">
         <v>1</v>
       </c>
+      <c r="T361" t="inlineStr"/>
     </row>
     <row r="362">
       <c r="A362" t="n">
@@ -18670,6 +19035,7 @@
       <c r="S362" t="n">
         <v>1</v>
       </c>
+      <c r="T362" t="inlineStr"/>
     </row>
     <row r="363">
       <c r="A363" t="n">
@@ -18719,6 +19085,7 @@
       <c r="S363" t="n">
         <v>1</v>
       </c>
+      <c r="T363" t="inlineStr"/>
     </row>
     <row r="364">
       <c r="A364" t="n">
@@ -18768,6 +19135,7 @@
       <c r="S364" t="n">
         <v>1</v>
       </c>
+      <c r="T364" t="inlineStr"/>
     </row>
     <row r="365">
       <c r="A365" t="n">
@@ -18817,6 +19185,7 @@
       <c r="S365" t="n">
         <v>1</v>
       </c>
+      <c r="T365" t="inlineStr"/>
     </row>
     <row r="366">
       <c r="A366" t="n">
@@ -18866,6 +19235,7 @@
       <c r="S366" t="n">
         <v>1</v>
       </c>
+      <c r="T366" t="inlineStr"/>
     </row>
     <row r="367">
       <c r="A367" t="n">
@@ -18915,6 +19285,7 @@
       <c r="S367" t="n">
         <v>1</v>
       </c>
+      <c r="T367" t="inlineStr"/>
     </row>
     <row r="368">
       <c r="A368" t="n">
@@ -18964,6 +19335,7 @@
       <c r="S368" t="n">
         <v>1</v>
       </c>
+      <c r="T368" t="inlineStr"/>
     </row>
     <row r="369">
       <c r="A369" t="n">
@@ -19013,6 +19385,7 @@
       <c r="S369" t="n">
         <v>1</v>
       </c>
+      <c r="T369" t="inlineStr"/>
     </row>
     <row r="370">
       <c r="A370" t="n">
@@ -19062,6 +19435,7 @@
       <c r="S370" t="n">
         <v>1</v>
       </c>
+      <c r="T370" t="inlineStr"/>
     </row>
     <row r="371">
       <c r="A371" t="n">
@@ -19111,6 +19485,7 @@
       <c r="S371" t="n">
         <v>1</v>
       </c>
+      <c r="T371" t="inlineStr"/>
     </row>
     <row r="372">
       <c r="A372" t="n">
@@ -19160,6 +19535,7 @@
       <c r="S372" t="n">
         <v>1</v>
       </c>
+      <c r="T372" t="inlineStr"/>
     </row>
     <row r="373">
       <c r="A373" t="n">
@@ -19209,6 +19585,7 @@
       <c r="S373" t="n">
         <v>1</v>
       </c>
+      <c r="T373" t="inlineStr"/>
     </row>
     <row r="374">
       <c r="A374" t="n">
@@ -19258,6 +19635,7 @@
       <c r="S374" t="n">
         <v>1</v>
       </c>
+      <c r="T374" t="inlineStr"/>
     </row>
     <row r="375">
       <c r="A375" t="n">
@@ -19307,6 +19685,7 @@
       <c r="S375" t="n">
         <v>1</v>
       </c>
+      <c r="T375" t="inlineStr"/>
     </row>
     <row r="376">
       <c r="A376" t="n">
@@ -19360,6 +19739,7 @@
       <c r="S376" t="n">
         <v>1</v>
       </c>
+      <c r="T376" t="inlineStr"/>
     </row>
     <row r="377">
       <c r="A377" t="n">
@@ -19413,6 +19793,7 @@
       <c r="S377" t="n">
         <v>1</v>
       </c>
+      <c r="T377" t="inlineStr"/>
     </row>
     <row r="378">
       <c r="A378" t="n">
@@ -19462,6 +19843,7 @@
       <c r="S378" t="n">
         <v>1</v>
       </c>
+      <c r="T378" t="inlineStr"/>
     </row>
     <row r="379">
       <c r="A379" t="n">
@@ -19511,6 +19893,7 @@
       <c r="S379" t="n">
         <v>1</v>
       </c>
+      <c r="T379" t="inlineStr"/>
     </row>
     <row r="380">
       <c r="A380" t="n">
@@ -19560,6 +19943,7 @@
       <c r="S380" t="n">
         <v>1</v>
       </c>
+      <c r="T380" t="inlineStr"/>
     </row>
     <row r="381">
       <c r="A381" t="n">
@@ -19613,6 +19997,7 @@
       <c r="S381" t="n">
         <v>1</v>
       </c>
+      <c r="T381" t="inlineStr"/>
     </row>
     <row r="382">
       <c r="A382" t="n">
@@ -19666,6 +20051,7 @@
       <c r="S382" t="n">
         <v>1</v>
       </c>
+      <c r="T382" t="inlineStr"/>
     </row>
     <row r="383">
       <c r="A383" t="n">
@@ -19719,6 +20105,7 @@
       <c r="S383" t="n">
         <v>1</v>
       </c>
+      <c r="T383" t="inlineStr"/>
     </row>
     <row r="384">
       <c r="A384" t="n">
@@ -19772,6 +20159,7 @@
       <c r="S384" t="n">
         <v>1</v>
       </c>
+      <c r="T384" t="inlineStr"/>
     </row>
     <row r="385">
       <c r="A385" t="n">
@@ -19825,6 +20213,7 @@
       <c r="S385" t="n">
         <v>1</v>
       </c>
+      <c r="T385" t="inlineStr"/>
     </row>
     <row r="386">
       <c r="A386" t="n">
@@ -19878,6 +20267,7 @@
       <c r="S386" t="n">
         <v>1</v>
       </c>
+      <c r="T386" t="inlineStr"/>
     </row>
     <row r="387">
       <c r="A387" t="n">
@@ -19931,6 +20321,7 @@
       <c r="S387" t="n">
         <v>1</v>
       </c>
+      <c r="T387" t="inlineStr"/>
     </row>
     <row r="388">
       <c r="A388" t="n">
@@ -19980,6 +20371,7 @@
       <c r="S388" t="n">
         <v>1</v>
       </c>
+      <c r="T388" t="inlineStr"/>
     </row>
     <row r="389">
       <c r="A389" t="n">
@@ -20033,6 +20425,7 @@
       <c r="S389" t="n">
         <v>1</v>
       </c>
+      <c r="T389" t="inlineStr"/>
     </row>
     <row r="390">
       <c r="A390" t="n">
@@ -20086,6 +20479,7 @@
       <c r="S390" t="n">
         <v>1</v>
       </c>
+      <c r="T390" t="inlineStr"/>
     </row>
     <row r="391">
       <c r="A391" t="n">
@@ -20139,6 +20533,7 @@
       <c r="S391" t="n">
         <v>1</v>
       </c>
+      <c r="T391" t="inlineStr"/>
     </row>
     <row r="392">
       <c r="A392" t="n">
@@ -20192,6 +20587,7 @@
       <c r="S392" t="n">
         <v>1</v>
       </c>
+      <c r="T392" t="inlineStr"/>
     </row>
     <row r="393">
       <c r="A393" t="n">
@@ -20245,6 +20641,7 @@
       <c r="S393" t="n">
         <v>1</v>
       </c>
+      <c r="T393" t="inlineStr"/>
     </row>
     <row r="394">
       <c r="A394" t="n">
@@ -20298,6 +20695,7 @@
       <c r="S394" t="n">
         <v>1</v>
       </c>
+      <c r="T394" t="inlineStr"/>
     </row>
     <row r="395">
       <c r="A395" t="n">
@@ -20351,6 +20749,7 @@
       <c r="S395" t="n">
         <v>1</v>
       </c>
+      <c r="T395" t="inlineStr"/>
     </row>
     <row r="396">
       <c r="A396" t="n">
@@ -20404,6 +20803,7 @@
       <c r="S396" t="n">
         <v>1</v>
       </c>
+      <c r="T396" t="inlineStr"/>
     </row>
     <row r="397">
       <c r="A397" t="n">
@@ -20457,6 +20857,7 @@
       <c r="S397" t="n">
         <v>1</v>
       </c>
+      <c r="T397" t="inlineStr"/>
     </row>
     <row r="398">
       <c r="A398" t="n">
@@ -20506,6 +20907,7 @@
       <c r="S398" t="n">
         <v>1</v>
       </c>
+      <c r="T398" t="inlineStr"/>
     </row>
     <row r="399">
       <c r="A399" t="n">
@@ -20559,6 +20961,7 @@
       <c r="S399" t="n">
         <v>1</v>
       </c>
+      <c r="T399" t="inlineStr"/>
     </row>
     <row r="400">
       <c r="A400" t="n">
@@ -20612,6 +21015,7 @@
       <c r="S400" t="n">
         <v>1</v>
       </c>
+      <c r="T400" t="inlineStr"/>
     </row>
     <row r="401">
       <c r="A401" t="n">
@@ -20665,6 +21069,7 @@
       <c r="S401" t="n">
         <v>1</v>
       </c>
+      <c r="T401" t="inlineStr"/>
     </row>
     <row r="402">
       <c r="A402" t="n">
@@ -20718,6 +21123,7 @@
       <c r="S402" t="n">
         <v>1</v>
       </c>
+      <c r="T402" t="inlineStr"/>
     </row>
     <row r="403">
       <c r="A403" t="n">
@@ -20771,6 +21177,7 @@
       <c r="S403" t="n">
         <v>1</v>
       </c>
+      <c r="T403" t="inlineStr"/>
     </row>
     <row r="404">
       <c r="A404" t="n">
@@ -20824,6 +21231,7 @@
       <c r="S404" t="n">
         <v>1</v>
       </c>
+      <c r="T404" t="inlineStr"/>
     </row>
     <row r="405">
       <c r="A405" t="n">
@@ -20877,6 +21285,7 @@
       <c r="S405" t="n">
         <v>1</v>
       </c>
+      <c r="T405" t="inlineStr"/>
     </row>
     <row r="406">
       <c r="A406" t="n">
@@ -20930,6 +21339,7 @@
       <c r="S406" t="n">
         <v>1</v>
       </c>
+      <c r="T406" t="inlineStr"/>
     </row>
     <row r="407">
       <c r="A407" t="n">
@@ -20983,6 +21393,7 @@
       <c r="S407" t="n">
         <v>0</v>
       </c>
+      <c r="T407" t="inlineStr"/>
     </row>
     <row r="408">
       <c r="A408" t="n">
@@ -21028,6 +21439,7 @@
       <c r="S408" t="n">
         <v>0</v>
       </c>
+      <c r="T408" t="inlineStr"/>
     </row>
     <row r="409">
       <c r="A409" t="n">
@@ -21073,6 +21485,7 @@
       <c r="S409" t="n">
         <v>0</v>
       </c>
+      <c r="T409" t="inlineStr"/>
     </row>
     <row r="410">
       <c r="A410" t="n">
@@ -21118,6 +21531,7 @@
       <c r="S410" t="n">
         <v>1</v>
       </c>
+      <c r="T410" t="inlineStr"/>
     </row>
     <row r="411">
       <c r="A411" t="n">
@@ -21163,6 +21577,7 @@
       <c r="S411" t="n">
         <v>1</v>
       </c>
+      <c r="T411" t="inlineStr"/>
     </row>
     <row r="412">
       <c r="A412" t="n">
@@ -21208,6 +21623,7 @@
       <c r="S412" t="n">
         <v>0</v>
       </c>
+      <c r="T412" t="inlineStr"/>
     </row>
     <row r="413">
       <c r="A413" t="n">
@@ -21253,6 +21669,7 @@
       <c r="S413" t="n">
         <v>0</v>
       </c>
+      <c r="T413" t="inlineStr"/>
     </row>
     <row r="414">
       <c r="A414" t="n">
@@ -21298,6 +21715,7 @@
       <c r="S414" t="n">
         <v>0</v>
       </c>
+      <c r="T414" t="inlineStr"/>
     </row>
     <row r="415">
       <c r="A415" t="n">
@@ -21343,6 +21761,7 @@
       <c r="S415" t="n">
         <v>1</v>
       </c>
+      <c r="T415" t="inlineStr"/>
     </row>
     <row r="416">
       <c r="A416" t="n">
@@ -21388,6 +21807,7 @@
       <c r="S416" t="n">
         <v>0</v>
       </c>
+      <c r="T416" t="inlineStr"/>
     </row>
     <row r="417">
       <c r="A417" t="n">
@@ -21403,7 +21823,7 @@
       <c r="E417" t="inlineStr"/>
       <c r="F417" t="inlineStr">
         <is>
-          <t>세척제</t>
+          <t>PT 세척제</t>
         </is>
       </c>
       <c r="G417" t="inlineStr"/>
@@ -21437,6 +21857,7 @@
       <c r="S417" t="n">
         <v>0</v>
       </c>
+      <c r="T417" t="inlineStr"/>
     </row>
     <row r="418">
       <c r="A418" t="n">
@@ -21452,7 +21873,7 @@
       <c r="E418" t="inlineStr"/>
       <c r="F418" t="inlineStr">
         <is>
-          <t>침투제</t>
+          <t>PT 침투제</t>
         </is>
       </c>
       <c r="G418" t="inlineStr"/>
@@ -21486,6 +21907,7 @@
       <c r="S418" t="n">
         <v>0</v>
       </c>
+      <c r="T418" t="inlineStr"/>
     </row>
     <row r="419">
       <c r="A419" t="n">
@@ -21501,7 +21923,7 @@
       <c r="E419" t="inlineStr"/>
       <c r="F419" t="inlineStr">
         <is>
-          <t>현상제</t>
+          <t>PT 현상제</t>
         </is>
       </c>
       <c r="G419" t="inlineStr"/>
@@ -21535,6 +21957,7 @@
       <c r="S419" t="n">
         <v>0</v>
       </c>
+      <c r="T419" t="inlineStr"/>
     </row>
     <row r="420">
       <c r="A420" t="n">
@@ -21588,6 +22011,7 @@
       <c r="S420" t="n">
         <v>0</v>
       </c>
+      <c r="T420" t="inlineStr"/>
     </row>
     <row r="421">
       <c r="A421" t="n">
@@ -21641,6 +22065,7 @@
       <c r="S421" t="n">
         <v>0</v>
       </c>
+      <c r="T421" t="inlineStr"/>
     </row>
     <row r="422">
       <c r="A422" t="n">
@@ -21694,6 +22119,7 @@
       <c r="S422" t="n">
         <v>0</v>
       </c>
+      <c r="T422" t="inlineStr"/>
     </row>
     <row r="423">
       <c r="A423" t="n">
@@ -21747,6 +22173,7 @@
       <c r="S423" t="n">
         <v>0</v>
       </c>
+      <c r="T423" t="inlineStr"/>
     </row>
     <row r="424">
       <c r="A424" t="n">
@@ -21800,6 +22227,7 @@
       <c r="S424" t="n">
         <v>0</v>
       </c>
+      <c r="T424" t="inlineStr"/>
     </row>
     <row r="425">
       <c r="A425" t="n">
@@ -21853,6 +22281,7 @@
       <c r="S425" t="n">
         <v>0</v>
       </c>
+      <c r="T425" t="inlineStr"/>
     </row>
     <row r="426">
       <c r="A426" t="n">
@@ -21906,6 +22335,7 @@
       <c r="S426" t="n">
         <v>1</v>
       </c>
+      <c r="T426" t="inlineStr"/>
     </row>
     <row r="427">
       <c r="A427" t="n">
@@ -21959,6 +22389,7 @@
       <c r="S427" t="n">
         <v>0</v>
       </c>
+      <c r="T427" t="inlineStr"/>
     </row>
     <row r="428">
       <c r="A428" t="n">
@@ -22012,6 +22443,7 @@
       <c r="S428" t="n">
         <v>0</v>
       </c>
+      <c r="T428" t="inlineStr"/>
     </row>
     <row r="429">
       <c r="A429" t="n">
@@ -22065,6 +22497,7 @@
       <c r="S429" t="n">
         <v>0</v>
       </c>
+      <c r="T429" t="inlineStr"/>
     </row>
     <row r="430">
       <c r="A430" t="n">
@@ -22117,6 +22550,169 @@
       </c>
       <c r="S430" t="n">
         <v>1</v>
+      </c>
+      <c r="T430" t="inlineStr"/>
+    </row>
+    <row r="431">
+      <c r="A431" t="n">
+        <v>433</v>
+      </c>
+      <c r="B431" t="inlineStr"/>
+      <c r="C431" t="inlineStr"/>
+      <c r="D431" t="inlineStr">
+        <is>
+          <t>MT약품</t>
+        </is>
+      </c>
+      <c r="E431" t="inlineStr">
+        <is>
+          <t>현장</t>
+        </is>
+      </c>
+      <c r="F431" t="inlineStr">
+        <is>
+          <t>MT 흑색자분</t>
+        </is>
+      </c>
+      <c r="G431" t="inlineStr">
+        <is>
+          <t>자동등록</t>
+        </is>
+      </c>
+      <c r="H431" t="inlineStr"/>
+      <c r="I431" t="inlineStr"/>
+      <c r="J431" t="inlineStr"/>
+      <c r="K431" t="n">
+        <v>0</v>
+      </c>
+      <c r="L431" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="M431" t="n">
+        <v>0</v>
+      </c>
+      <c r="N431" t="inlineStr"/>
+      <c r="O431" t="inlineStr"/>
+      <c r="P431" t="inlineStr"/>
+      <c r="Q431" t="n">
+        <v>10</v>
+      </c>
+      <c r="R431" t="n">
+        <v>0</v>
+      </c>
+      <c r="S431" t="n">
+        <v>1</v>
+      </c>
+      <c r="T431" t="inlineStr"/>
+    </row>
+    <row r="432">
+      <c r="A432" t="n">
+        <v>434</v>
+      </c>
+      <c r="B432" t="inlineStr"/>
+      <c r="C432" t="inlineStr"/>
+      <c r="D432" t="inlineStr">
+        <is>
+          <t>MT약품</t>
+        </is>
+      </c>
+      <c r="E432" t="inlineStr">
+        <is>
+          <t>현장</t>
+        </is>
+      </c>
+      <c r="F432" t="inlineStr">
+        <is>
+          <t>MT 백색페인트</t>
+        </is>
+      </c>
+      <c r="G432" t="inlineStr">
+        <is>
+          <t>자동등록</t>
+        </is>
+      </c>
+      <c r="H432" t="inlineStr"/>
+      <c r="I432" t="inlineStr"/>
+      <c r="J432" t="inlineStr"/>
+      <c r="K432" t="n">
+        <v>0</v>
+      </c>
+      <c r="L432" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="M432" t="n">
+        <v>0</v>
+      </c>
+      <c r="N432" t="inlineStr"/>
+      <c r="O432" t="inlineStr"/>
+      <c r="P432" t="inlineStr"/>
+      <c r="Q432" t="n">
+        <v>10</v>
+      </c>
+      <c r="R432" t="n">
+        <v>0</v>
+      </c>
+      <c r="S432" t="n">
+        <v>1</v>
+      </c>
+      <c r="T432" t="inlineStr"/>
+    </row>
+    <row r="433">
+      <c r="A433" t="n">
+        <v>432</v>
+      </c>
+      <c r="B433" t="inlineStr"/>
+      <c r="C433" t="inlineStr"/>
+      <c r="D433" t="inlineStr">
+        <is>
+          <t>MT약품</t>
+        </is>
+      </c>
+      <c r="E433" t="inlineStr">
+        <is>
+          <t>현장</t>
+        </is>
+      </c>
+      <c r="F433" t="inlineStr"/>
+      <c r="G433" t="inlineStr">
+        <is>
+          <t>자동등록</t>
+        </is>
+      </c>
+      <c r="H433" t="inlineStr"/>
+      <c r="I433" t="inlineStr"/>
+      <c r="J433" t="inlineStr"/>
+      <c r="K433" t="n">
+        <v>0</v>
+      </c>
+      <c r="L433" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="M433" t="n">
+        <v>0</v>
+      </c>
+      <c r="N433" t="inlineStr"/>
+      <c r="O433" t="inlineStr"/>
+      <c r="P433" t="inlineStr"/>
+      <c r="Q433" t="n">
+        <v>0</v>
+      </c>
+      <c r="R433" t="n">
+        <v>0</v>
+      </c>
+      <c r="S433" t="n">
+        <v>0</v>
+      </c>
+      <c r="T433" t="inlineStr">
+        <is>
+          <t>사용가능</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -22130,7 +22726,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W3"/>
+  <dimension ref="A1:W5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22375,6 +22971,100 @@
       <c r="U3" t="inlineStr"/>
       <c r="V3" t="inlineStr"/>
       <c r="W3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="n">
+        <v>46128.89430152778</v>
+      </c>
+      <c r="B4" t="n">
+        <v>433</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>-1</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>K-1 PJT 현장 사용 (자동 차감)</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>부장 주진철, 대리 우명광</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>K-1 PJT</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr"/>
+      <c r="R4" t="inlineStr"/>
+      <c r="S4" t="inlineStr"/>
+      <c r="T4" t="inlineStr"/>
+      <c r="U4" t="inlineStr"/>
+      <c r="V4" t="inlineStr"/>
+      <c r="W4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="n">
+        <v>46128.89430152778</v>
+      </c>
+      <c r="B5" t="n">
+        <v>434</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>-1</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>K-1 PJT 현장 사용 (자동 차감)</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>부장 주진철, 대리 우명광</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>K-1 PJT</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr"/>
+      <c r="Q5" t="inlineStr"/>
+      <c r="R5" t="inlineStr"/>
+      <c r="S5" t="inlineStr"/>
+      <c r="T5" t="inlineStr"/>
+      <c r="U5" t="inlineStr"/>
+      <c r="V5" t="inlineStr"/>
+      <c r="W5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -22448,7 +23138,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CB5"/>
+  <dimension ref="A1:CB6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23593,6 +24283,188 @@
       <c r="CA5" t="inlineStr"/>
       <c r="CB5" t="inlineStr"/>
     </row>
+    <row r="6">
+      <c r="A6" s="1" t="n">
+        <v>46128</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>K-1 PJT</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>432</v>
+      </c>
+      <c r="D6" t="n">
+        <v>50</v>
+      </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" s="1" t="n">
+        <v>46139.8943015162</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>부장 주진철</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>YOKE AC-NW1301154</t>
+        </is>
+      </c>
+      <c r="P6" t="n">
+        <v>50</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>4300</v>
+      </c>
+      <c r="R6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T6" t="n">
+        <v>215000</v>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>MT</t>
+        </is>
+      </c>
+      <c r="V6" t="n">
+        <v>0</v>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>(주간) 09:00~18:00</t>
+        </is>
+      </c>
+      <c r="X6" t="inlineStr"/>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>대리 우명광</t>
+        </is>
+      </c>
+      <c r="Z6" t="inlineStr">
+        <is>
+          <t>(주간) 09:00~18:00</t>
+        </is>
+      </c>
+      <c r="AA6" t="inlineStr"/>
+      <c r="AB6" t="inlineStr"/>
+      <c r="AC6" t="inlineStr"/>
+      <c r="AD6" t="inlineStr"/>
+      <c r="AE6" t="inlineStr"/>
+      <c r="AF6" t="inlineStr"/>
+      <c r="AG6" t="inlineStr"/>
+      <c r="AH6" t="inlineStr"/>
+      <c r="AI6" t="inlineStr"/>
+      <c r="AJ6" t="inlineStr"/>
+      <c r="AK6" t="inlineStr"/>
+      <c r="AL6" t="inlineStr"/>
+      <c r="AM6" t="inlineStr"/>
+      <c r="AN6" t="inlineStr"/>
+      <c r="AO6" t="inlineStr"/>
+      <c r="AP6" t="inlineStr"/>
+      <c r="AQ6" t="inlineStr"/>
+      <c r="AR6" t="inlineStr"/>
+      <c r="AS6" t="inlineStr"/>
+      <c r="AT6" t="inlineStr"/>
+      <c r="AU6" t="inlineStr"/>
+      <c r="AV6" t="inlineStr"/>
+      <c r="AW6" t="inlineStr"/>
+      <c r="AX6" t="inlineStr"/>
+      <c r="AY6" t="inlineStr"/>
+      <c r="AZ6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA6" t="n">
+        <v>1</v>
+      </c>
+      <c r="BB6" t="n">
+        <v>1</v>
+      </c>
+      <c r="BC6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH6" t="inlineStr">
+        <is>
+          <t>스타렉스81루5100</t>
+        </is>
+      </c>
+      <c r="BI6" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="BJ6" t="inlineStr">
+        <is>
+          <t>out_exterior:양호|out_cleanliness:양호|out_cleaning:함|in_exterior:양호|in_cleanliness:양호|in_cleaning:함</t>
+        </is>
+      </c>
+      <c r="BK6" t="inlineStr"/>
+      <c r="BL6" t="inlineStr"/>
+      <c r="BM6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN6" t="inlineStr"/>
+      <c r="BO6" t="inlineStr">
+        <is>
+          <t>롯데건설</t>
+        </is>
+      </c>
+      <c r="BP6" t="inlineStr"/>
+      <c r="BQ6" t="inlineStr"/>
+      <c r="BR6" t="inlineStr"/>
+      <c r="BS6" t="inlineStr"/>
+      <c r="BT6" t="inlineStr"/>
+      <c r="BU6" t="inlineStr"/>
+      <c r="BV6" t="inlineStr"/>
+      <c r="BW6" t="inlineStr"/>
+      <c r="BX6" t="inlineStr"/>
+      <c r="BY6" t="inlineStr">
+        <is>
+          <t>PIPE</t>
+        </is>
+      </c>
+      <c r="BZ6" t="inlineStr"/>
+      <c r="CA6" t="inlineStr"/>
+      <c r="CB6" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>